<commit_message>
Senegal Wave 1 FIES logic added.
In Mongolia and Turkmenistan tab plans Preparation Files were added as a sheet and corresponding R files were removed.
</commit_message>
<xml_diff>
--- a/Senegal (2026) Wave 1/SEN MICSPlus 2026 Wave1_TabPlan_20261019.xlsx
+++ b/Senegal (2026) Wave 1/SEN MICSPlus 2026 Wave1_TabPlan_20261019.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11011"/>
   <workbookPr filterPrivacy="1" updateLinks="always" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{505C068C-4D50-A740-B757-F464F220966A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4120" yWindow="660" windowWidth="26320" windowHeight="21680" tabRatio="861" firstSheet="12" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4120" yWindow="660" windowWidth="26320" windowHeight="21680" tabRatio="861" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IDX" sheetId="49" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2287" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2288" uniqueCount="809">
   <si>
     <t>Survey and sample characteristics</t>
   </si>
@@ -3324,6 +3324,27 @@
 ea43more %in% c(1) |
 (between(RS2B, 5, 14) &amp; hhc21more %in% c(1)) |
 tothaz %in% c(1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Extra table: FIES ----------------------------------------------------
+tables_extra &lt;- c("4.1")
+extra_tables_dict &lt;- list(
+  "4.1" = "tb_41"
+)
+# Preserve prepared datasets in case the FIES script overwrites them.
+hh_before_fies &lt;- hh
+hl_before_fies &lt;- hl
+# Senegal FIES script: country code SEN, Wave 1, Table 4.1.
+source(
+  file.path(path_fies, "SEN MICSPlus Wave1 - Table 4.1_Script.R"),
+  local = TRUE
+)
+# If the script returns res.df rather than tb_41,
+# insert the conversion of its results into tb_41 here.
+stopifnot(exists("tb_41", inherits = FALSE))
+hh &lt;- hh_before_fies
+hl &lt;- hl_before_fies
+</t>
   </si>
 </sst>
 </file>
@@ -8096,6 +8117,63 @@
     <xf numFmtId="0" fontId="45" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -8505,24 +8583,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8540,18 +8600,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -8573,36 +8624,6 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -8702,6 +8723,30 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="891" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="891" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -8709,30 +8754,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="891" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="891" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="891" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -13446,20 +13467,20 @@
   <sheetData>
     <row r="1" spans="2:13" ht="6" customHeight="1"/>
     <row r="2" spans="2:13" s="210" customFormat="1" ht="13">
-      <c r="B2" s="556" t="s">
+      <c r="B2" s="575" t="s">
         <v>764</v>
       </c>
-      <c r="C2" s="557"/>
-      <c r="D2" s="557"/>
-      <c r="E2" s="557"/>
-      <c r="F2" s="557"/>
-      <c r="G2" s="557"/>
-      <c r="H2" s="557"/>
-      <c r="I2" s="557"/>
-      <c r="J2" s="557"/>
-      <c r="K2" s="557"/>
-      <c r="L2" s="557"/>
-      <c r="M2" s="558"/>
+      <c r="C2" s="576"/>
+      <c r="D2" s="576"/>
+      <c r="E2" s="576"/>
+      <c r="F2" s="576"/>
+      <c r="G2" s="576"/>
+      <c r="H2" s="576"/>
+      <c r="I2" s="576"/>
+      <c r="J2" s="576"/>
+      <c r="K2" s="576"/>
+      <c r="L2" s="576"/>
+      <c r="M2" s="577"/>
     </row>
     <row r="3" spans="2:13" s="210" customFormat="1" ht="13">
       <c r="B3" s="549" t="s">
@@ -13557,14 +13578,14 @@
       <c r="M9" s="17"/>
     </row>
     <row r="10" spans="2:13" ht="12" customHeight="1">
-      <c r="B10" s="559" t="str">
+      <c r="B10" s="578" t="str">
         <f>'1.1a'!A1</f>
         <v>Table 1.1a Response rates (after substitution, unweighted)</v>
       </c>
-      <c r="C10" s="560"/>
-      <c r="D10" s="560"/>
-      <c r="E10" s="560"/>
-      <c r="F10" s="560"/>
+      <c r="C10" s="579"/>
+      <c r="D10" s="579"/>
+      <c r="E10" s="579"/>
+      <c r="F10" s="579"/>
       <c r="H10" s="68" t="str">
         <f>'5.1'!A1</f>
         <v>Table 5.1 Child discipline</v>
@@ -13576,14 +13597,14 @@
       <c r="M10" s="17"/>
     </row>
     <row r="11" spans="2:13" ht="12" customHeight="1">
-      <c r="B11" s="559" t="str">
+      <c r="B11" s="578" t="str">
         <f>'1.1b'!A1</f>
         <v>Table 1.1b Response rates (before substitution, unweighted)</v>
       </c>
-      <c r="C11" s="560"/>
-      <c r="D11" s="560"/>
-      <c r="E11" s="560"/>
-      <c r="F11" s="560"/>
+      <c r="C11" s="579"/>
+      <c r="D11" s="579"/>
+      <c r="E11" s="579"/>
+      <c r="F11" s="579"/>
       <c r="H11" s="68" t="str">
         <f>'5.2'!A1</f>
         <v xml:space="preserve">Table 5.2 Attitudes toward physical punishment </v>
@@ -13595,14 +13616,14 @@
       <c r="M11" s="17"/>
     </row>
     <row r="12" spans="2:13" ht="12" customHeight="1">
-      <c r="B12" s="559" t="str">
+      <c r="B12" s="578" t="str">
         <f>'1.2'!A1</f>
         <v>Table 1.2 Average number of call attempts (unweighted)</v>
       </c>
-      <c r="C12" s="560"/>
-      <c r="D12" s="560"/>
-      <c r="E12" s="560"/>
-      <c r="F12" s="560"/>
+      <c r="C12" s="579"/>
+      <c r="D12" s="579"/>
+      <c r="E12" s="579"/>
+      <c r="F12" s="579"/>
       <c r="I12" s="68"/>
       <c r="J12" s="68"/>
       <c r="K12" s="68"/>
@@ -13610,14 +13631,14 @@
       <c r="M12" s="17"/>
     </row>
     <row r="13" spans="2:13" ht="12" customHeight="1">
-      <c r="B13" s="559" t="str">
+      <c r="B13" s="578" t="str">
         <f>'1.3'!A1</f>
         <v>Table 1.3 Number of call attempts (unweighted)</v>
       </c>
-      <c r="C13" s="560"/>
-      <c r="D13" s="560"/>
-      <c r="E13" s="560"/>
-      <c r="F13" s="560"/>
+      <c r="C13" s="579"/>
+      <c r="D13" s="579"/>
+      <c r="E13" s="579"/>
+      <c r="F13" s="579"/>
       <c r="H13" s="72" t="s">
         <v>2</v>
       </c>
@@ -13628,14 +13649,14 @@
       <c r="M13" s="17"/>
     </row>
     <row r="14" spans="2:13" ht="12" customHeight="1">
-      <c r="B14" s="559" t="str">
+      <c r="B14" s="578" t="str">
         <f>'1.4'!A1</f>
         <v>Table 1.4 Duration of interviews (unweighted)</v>
       </c>
-      <c r="C14" s="560"/>
-      <c r="D14" s="560"/>
-      <c r="E14" s="560"/>
-      <c r="F14" s="560"/>
+      <c r="C14" s="579"/>
+      <c r="D14" s="579"/>
+      <c r="E14" s="579"/>
+      <c r="F14" s="579"/>
       <c r="H14" s="68" t="str">
         <f>'6.1'!A1</f>
         <v>Table 6.1 Children's involvement in economic activities</v>
@@ -13647,14 +13668,14 @@
       <c r="M14" s="22"/>
     </row>
     <row r="15" spans="2:13" ht="12" customHeight="1">
-      <c r="B15" s="559" t="str">
+      <c r="B15" s="578" t="str">
         <f>'2.1'!A1</f>
         <v>Table 2.1 Housing characteristics</v>
       </c>
-      <c r="C15" s="560"/>
-      <c r="D15" s="560"/>
-      <c r="E15" s="560"/>
-      <c r="F15" s="560"/>
+      <c r="C15" s="579"/>
+      <c r="D15" s="579"/>
+      <c r="E15" s="579"/>
+      <c r="F15" s="579"/>
       <c r="H15" s="68" t="str">
         <f>'6.2'!A1</f>
         <v>Table 6.2 Children's involvement in household chores</v>
@@ -13666,14 +13687,14 @@
       <c r="M15" s="22"/>
     </row>
     <row r="16" spans="2:13" ht="12" customHeight="1">
-      <c r="B16" s="559" t="str">
+      <c r="B16" s="578" t="str">
         <f>'2.1a'!A1</f>
         <v>Table 2.1a Sources of electricity</v>
       </c>
-      <c r="C16" s="560"/>
-      <c r="D16" s="560"/>
-      <c r="E16" s="560"/>
-      <c r="F16" s="560"/>
+      <c r="C16" s="579"/>
+      <c r="D16" s="579"/>
+      <c r="E16" s="579"/>
+      <c r="F16" s="579"/>
       <c r="H16" s="68" t="str">
         <f>'6.3'!A1</f>
         <v>Table 6.3 Child labour</v>
@@ -13685,14 +13706,14 @@
       <c r="M16" s="22"/>
     </row>
     <row r="17" spans="2:13" ht="12" customHeight="1">
-      <c r="B17" s="559" t="str">
+      <c r="B17" s="578" t="str">
         <f>'2.1b'!A1</f>
         <v>Table 2.1b Household and personal assets</v>
       </c>
-      <c r="C17" s="560"/>
-      <c r="D17" s="560"/>
-      <c r="E17" s="560"/>
-      <c r="F17" s="560"/>
+      <c r="C17" s="579"/>
+      <c r="D17" s="579"/>
+      <c r="E17" s="579"/>
+      <c r="F17" s="579"/>
       <c r="G17" s="68"/>
       <c r="H17" s="68" t="str">
         <f>'6.4'!A1</f>
@@ -13938,41 +13959,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="561" t="s">
+      <c r="A1" s="580" t="s">
         <v>524</v>
       </c>
-      <c r="B1" s="562"/>
-      <c r="C1" s="562"/>
-      <c r="D1" s="562"/>
-      <c r="E1" s="563"/>
+      <c r="B1" s="581"/>
+      <c r="C1" s="581"/>
+      <c r="D1" s="581"/>
+      <c r="E1" s="582"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="611" t="s">
+      <c r="A2" s="630" t="s">
         <v>534</v>
       </c>
-      <c r="B2" s="612"/>
-      <c r="C2" s="612"/>
-      <c r="D2" s="612"/>
-      <c r="E2" s="613"/>
+      <c r="B2" s="631"/>
+      <c r="C2" s="631"/>
+      <c r="D2" s="631"/>
+      <c r="E2" s="632"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="614"/>
+      <c r="A3" s="633"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="615" t="s">
+      <c r="C3" s="634" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="616" t="s">
+      <c r="D3" s="635" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="617"/>
+      <c r="E3" s="636"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="607"/>
+      <c r="C4" s="626"/>
       <c r="D4" s="102" t="s">
         <v>11</v>
       </c>
@@ -14132,13 +14153,13 @@
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" s="19" customFormat="1" ht="23" customHeight="1">
-      <c r="A19" s="608" t="s">
+      <c r="A19" s="627" t="s">
         <v>547</v>
       </c>
-      <c r="B19" s="609"/>
-      <c r="C19" s="609"/>
-      <c r="D19" s="609"/>
-      <c r="E19" s="610"/>
+      <c r="B19" s="628"/>
+      <c r="C19" s="628"/>
+      <c r="D19" s="628"/>
+      <c r="E19" s="629"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
@@ -14300,44 +14321,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="561" t="s">
+      <c r="A1" s="580" t="s">
         <v>548</v>
       </c>
-      <c r="B1" s="562"/>
-      <c r="C1" s="562"/>
-      <c r="D1" s="562"/>
-      <c r="E1" s="563"/>
+      <c r="B1" s="581"/>
+      <c r="C1" s="581"/>
+      <c r="D1" s="581"/>
+      <c r="E1" s="582"/>
       <c r="F1" s="32"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="564" t="s">
+      <c r="A2" s="583" t="s">
         <v>144</v>
       </c>
-      <c r="B2" s="565"/>
-      <c r="C2" s="565"/>
-      <c r="D2" s="565"/>
-      <c r="E2" s="566"/>
+      <c r="B2" s="584"/>
+      <c r="C2" s="584"/>
+      <c r="D2" s="584"/>
+      <c r="E2" s="585"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="567"/>
+      <c r="A3" s="586"/>
       <c r="B3" s="100"/>
-      <c r="C3" s="569" t="s">
+      <c r="C3" s="588" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="570" t="s">
+      <c r="D3" s="589" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="571"/>
+      <c r="E3" s="590"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="607"/>
+      <c r="C4" s="626"/>
       <c r="D4" s="102" t="s">
         <v>11</v>
       </c>
@@ -15250,58 +15271,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>551</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="611"/>
       <c r="J1" s="89"/>
       <c r="K1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="11.25" customHeight="1">
-      <c r="A2" s="618" t="s">
+      <c r="A2" s="637" t="s">
         <v>196</v>
       </c>
-      <c r="B2" s="619"/>
-      <c r="C2" s="619"/>
-      <c r="D2" s="619"/>
-      <c r="E2" s="619"/>
-      <c r="F2" s="619"/>
-      <c r="G2" s="619"/>
-      <c r="H2" s="620"/>
-      <c r="I2" s="621"/>
+      <c r="B2" s="638"/>
+      <c r="C2" s="638"/>
+      <c r="D2" s="638"/>
+      <c r="E2" s="638"/>
+      <c r="F2" s="638"/>
+      <c r="G2" s="638"/>
+      <c r="H2" s="639"/>
+      <c r="I2" s="640"/>
       <c r="J2" s="89"/>
       <c r="K2" s="89"/>
     </row>
     <row r="3" spans="1:11" ht="11.25" customHeight="1">
-      <c r="A3" s="622"/>
+      <c r="A3" s="641"/>
       <c r="B3" s="81"/>
-      <c r="C3" s="624" t="s">
+      <c r="C3" s="643" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="624"/>
-      <c r="E3" s="624"/>
-      <c r="F3" s="624"/>
-      <c r="G3" s="624"/>
-      <c r="H3" s="625" t="s">
+      <c r="D3" s="643"/>
+      <c r="E3" s="643"/>
+      <c r="F3" s="643"/>
+      <c r="G3" s="643"/>
+      <c r="H3" s="644" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="602" t="s">
+      <c r="I3" s="621" t="s">
         <v>115</v>
       </c>
       <c r="J3" s="20"/>
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:11" ht="14.5" customHeight="1">
-      <c r="A4" s="623"/>
+      <c r="A4" s="642"/>
       <c r="B4" s="82"/>
       <c r="C4" s="80" t="s">
         <v>198</v>
@@ -15318,8 +15339,8 @@
       <c r="G4" s="80" t="s">
         <v>202</v>
       </c>
-      <c r="H4" s="626"/>
-      <c r="I4" s="603"/>
+      <c r="H4" s="645"/>
+      <c r="I4" s="622"/>
       <c r="J4" s="20"/>
       <c r="K4" s="20"/>
     </row>
@@ -15789,44 +15810,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="611"/>
       <c r="F1" s="32"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="11.25" customHeight="1">
-      <c r="A2" s="593" t="s">
+      <c r="A2" s="612" t="s">
         <v>211</v>
       </c>
-      <c r="B2" s="594"/>
-      <c r="C2" s="594"/>
-      <c r="D2" s="595"/>
-      <c r="E2" s="596"/>
+      <c r="B2" s="613"/>
+      <c r="C2" s="613"/>
+      <c r="D2" s="614"/>
+      <c r="E2" s="615"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="614"/>
+      <c r="A3" s="633"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="615" t="s">
+      <c r="C3" s="634" t="s">
         <v>212</v>
       </c>
-      <c r="D3" s="616" t="s">
+      <c r="D3" s="635" t="s">
         <v>142</v>
       </c>
-      <c r="E3" s="617"/>
+      <c r="E3" s="636"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="607"/>
+      <c r="C4" s="626"/>
       <c r="D4" s="102" t="s">
         <v>213</v>
       </c>
@@ -17009,31 +17030,31 @@
       <c r="N68" s="32"/>
     </row>
     <row r="69" spans="1:14" s="26" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A69" s="627" t="s">
+      <c r="A69" s="646" t="s">
         <v>588</v>
       </c>
-      <c r="B69" s="628"/>
-      <c r="C69" s="628"/>
-      <c r="D69" s="628"/>
-      <c r="E69" s="629"/>
+      <c r="B69" s="647"/>
+      <c r="C69" s="647"/>
+      <c r="D69" s="647"/>
+      <c r="E69" s="648"/>
     </row>
     <row r="70" spans="1:14" s="26" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A70" s="630" t="s">
+      <c r="A70" s="649" t="s">
         <v>589</v>
       </c>
-      <c r="B70" s="631"/>
-      <c r="C70" s="631"/>
-      <c r="D70" s="631"/>
-      <c r="E70" s="632"/>
+      <c r="B70" s="650"/>
+      <c r="C70" s="650"/>
+      <c r="D70" s="650"/>
+      <c r="E70" s="651"/>
     </row>
     <row r="71" spans="1:14" s="26" customFormat="1" ht="11">
-      <c r="A71" s="633" t="s">
+      <c r="A71" s="652" t="s">
         <v>587</v>
       </c>
-      <c r="B71" s="634"/>
-      <c r="C71" s="634"/>
-      <c r="D71" s="634"/>
-      <c r="E71" s="635"/>
+      <c r="B71" s="653"/>
+      <c r="C71" s="653"/>
+      <c r="D71" s="653"/>
+      <c r="E71" s="654"/>
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="32"/>
@@ -18037,18 +18058,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="15">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>249</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="611"/>
       <c r="K1" s="89"/>
       <c r="L1" s="86" t="s">
         <v>7</v>
@@ -18062,18 +18083,18 @@
       <c r="S1" s="32"/>
     </row>
     <row r="2" spans="1:19" ht="14">
-      <c r="A2" s="593" t="s">
+      <c r="A2" s="612" t="s">
         <v>250</v>
       </c>
-      <c r="B2" s="594"/>
-      <c r="C2" s="594"/>
-      <c r="D2" s="594"/>
-      <c r="E2" s="594"/>
-      <c r="F2" s="594"/>
-      <c r="G2" s="594"/>
-      <c r="H2" s="594"/>
-      <c r="I2" s="595"/>
-      <c r="J2" s="596"/>
+      <c r="B2" s="613"/>
+      <c r="C2" s="613"/>
+      <c r="D2" s="613"/>
+      <c r="E2" s="613"/>
+      <c r="F2" s="613"/>
+      <c r="G2" s="613"/>
+      <c r="H2" s="613"/>
+      <c r="I2" s="614"/>
+      <c r="J2" s="615"/>
       <c r="K2" s="89"/>
       <c r="L2" s="89"/>
       <c r="M2" s="32"/>
@@ -18085,27 +18106,27 @@
       <c r="S2" s="32"/>
     </row>
     <row r="3" spans="1:19" s="3" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="614"/>
+      <c r="A3" s="633"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="616" t="s">
+      <c r="C3" s="635" t="s">
         <v>251</v>
       </c>
-      <c r="D3" s="616"/>
+      <c r="D3" s="635"/>
       <c r="E3" s="101"/>
-      <c r="F3" s="616" t="s">
+      <c r="F3" s="635" t="s">
         <v>252</v>
       </c>
-      <c r="G3" s="616"/>
+      <c r="G3" s="635"/>
       <c r="H3" s="101"/>
-      <c r="I3" s="616" t="s">
+      <c r="I3" s="635" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="617"/>
+      <c r="J3" s="636"/>
       <c r="K3" s="20"/>
       <c r="L3" s="20"/>
     </row>
     <row r="4" spans="1:19" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="567"/>
+      <c r="A4" s="586"/>
       <c r="B4" s="100"/>
       <c r="C4" s="122" t="s">
         <v>64</v>
@@ -19098,16 +19119,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>291</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="611"/>
       <c r="I1" s="89"/>
       <c r="J1" s="86" t="s">
         <v>7</v>
@@ -19115,33 +19136,33 @@
       <c r="K1" s="21"/>
     </row>
     <row r="2" spans="1:11" ht="14">
-      <c r="A2" s="593" t="s">
+      <c r="A2" s="612" t="s">
         <v>292</v>
       </c>
-      <c r="B2" s="594"/>
-      <c r="C2" s="594"/>
-      <c r="D2" s="594"/>
-      <c r="E2" s="594"/>
-      <c r="F2" s="594"/>
-      <c r="G2" s="595"/>
-      <c r="H2" s="596"/>
+      <c r="B2" s="613"/>
+      <c r="C2" s="613"/>
+      <c r="D2" s="613"/>
+      <c r="E2" s="613"/>
+      <c r="F2" s="613"/>
+      <c r="G2" s="614"/>
+      <c r="H2" s="615"/>
       <c r="I2" s="89"/>
       <c r="J2" s="89"/>
       <c r="K2" s="21"/>
     </row>
     <row r="3" spans="1:11" ht="25.25" customHeight="1">
-      <c r="A3" s="614"/>
+      <c r="A3" s="633"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="616" t="s">
+      <c r="C3" s="635" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="616"/>
-      <c r="E3" s="616"/>
-      <c r="F3" s="616"/>
-      <c r="G3" s="640" t="s">
+      <c r="D3" s="635"/>
+      <c r="E3" s="635"/>
+      <c r="F3" s="635"/>
+      <c r="G3" s="659" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="642" t="s">
+      <c r="H3" s="661" t="s">
         <v>115</v>
       </c>
       <c r="I3" s="20"/>
@@ -19149,26 +19170,26 @@
       <c r="K3" s="21"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="567"/>
+      <c r="A4" s="586"/>
       <c r="B4" s="100"/>
-      <c r="C4" s="615" t="s">
+      <c r="C4" s="634" t="s">
         <v>294</v>
       </c>
-      <c r="D4" s="639" t="s">
+      <c r="D4" s="658" t="s">
         <v>295</v>
       </c>
-      <c r="E4" s="639"/>
-      <c r="F4" s="639"/>
-      <c r="G4" s="641"/>
-      <c r="H4" s="643"/>
+      <c r="E4" s="658"/>
+      <c r="F4" s="658"/>
+      <c r="G4" s="660"/>
+      <c r="H4" s="662"/>
       <c r="I4" s="20"/>
       <c r="J4" s="20"/>
       <c r="K4" s="21"/>
     </row>
     <row r="5" spans="1:11" ht="21.5" customHeight="1">
-      <c r="A5" s="568"/>
+      <c r="A5" s="587"/>
       <c r="B5" s="102"/>
-      <c r="C5" s="607"/>
+      <c r="C5" s="626"/>
       <c r="D5" s="103" t="s">
         <v>296</v>
       </c>
@@ -19178,8 +19199,8 @@
       <c r="F5" s="103" t="s">
         <v>298</v>
       </c>
-      <c r="G5" s="641"/>
-      <c r="H5" s="644"/>
+      <c r="G5" s="660"/>
+      <c r="H5" s="663"/>
       <c r="I5" s="20"/>
       <c r="J5" s="20"/>
       <c r="K5" s="21"/>
@@ -19424,16 +19445,16 @@
       <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="22.5" customHeight="1">
-      <c r="A19" s="636" t="s">
+      <c r="A19" s="655" t="s">
         <v>308</v>
       </c>
-      <c r="B19" s="637"/>
-      <c r="C19" s="637"/>
-      <c r="D19" s="637"/>
-      <c r="E19" s="637"/>
-      <c r="F19" s="637"/>
-      <c r="G19" s="637"/>
-      <c r="H19" s="638"/>
+      <c r="B19" s="656"/>
+      <c r="C19" s="656"/>
+      <c r="D19" s="656"/>
+      <c r="E19" s="656"/>
+      <c r="F19" s="656"/>
+      <c r="G19" s="656"/>
+      <c r="H19" s="657"/>
       <c r="I19" s="20"/>
       <c r="J19" s="88"/>
       <c r="K19" s="65"/>
@@ -19771,71 +19792,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15">
-      <c r="A1" s="647" t="s">
+      <c r="A1" s="666" t="s">
         <v>309</v>
       </c>
-      <c r="B1" s="648"/>
-      <c r="C1" s="648"/>
-      <c r="D1" s="648"/>
-      <c r="E1" s="648"/>
-      <c r="F1" s="648"/>
-      <c r="G1" s="648"/>
-      <c r="H1" s="648"/>
-      <c r="I1" s="648"/>
-      <c r="J1" s="648"/>
-      <c r="K1" s="648"/>
-      <c r="L1" s="649"/>
+      <c r="B1" s="667"/>
+      <c r="C1" s="667"/>
+      <c r="D1" s="667"/>
+      <c r="E1" s="667"/>
+      <c r="F1" s="667"/>
+      <c r="G1" s="667"/>
+      <c r="H1" s="667"/>
+      <c r="I1" s="667"/>
+      <c r="J1" s="667"/>
+      <c r="K1" s="667"/>
+      <c r="L1" s="668"/>
       <c r="M1" s="89"/>
       <c r="N1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="650" t="s">
+      <c r="A2" s="669" t="s">
         <v>599</v>
       </c>
-      <c r="B2" s="651"/>
-      <c r="C2" s="651"/>
-      <c r="D2" s="651"/>
-      <c r="E2" s="651"/>
-      <c r="F2" s="651"/>
-      <c r="G2" s="651"/>
-      <c r="H2" s="651"/>
-      <c r="I2" s="651"/>
-      <c r="J2" s="651"/>
-      <c r="K2" s="651"/>
-      <c r="L2" s="652"/>
+      <c r="B2" s="670"/>
+      <c r="C2" s="670"/>
+      <c r="D2" s="670"/>
+      <c r="E2" s="670"/>
+      <c r="F2" s="670"/>
+      <c r="G2" s="670"/>
+      <c r="H2" s="670"/>
+      <c r="I2" s="670"/>
+      <c r="J2" s="670"/>
+      <c r="K2" s="670"/>
+      <c r="L2" s="671"/>
       <c r="M2" s="89"/>
       <c r="N2" s="89"/>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" ht="11" customHeight="1">
-      <c r="A3" s="645"/>
+      <c r="A3" s="664"/>
       <c r="B3" s="322"/>
-      <c r="C3" s="658" t="s">
+      <c r="C3" s="677" t="s">
         <v>598</v>
       </c>
       <c r="D3" s="386"/>
-      <c r="E3" s="653" t="s">
+      <c r="E3" s="672" t="s">
         <v>597</v>
       </c>
-      <c r="F3" s="653"/>
-      <c r="G3" s="653"/>
-      <c r="H3" s="653"/>
-      <c r="I3" s="653"/>
-      <c r="J3" s="653"/>
-      <c r="K3" s="654" t="s">
+      <c r="F3" s="672"/>
+      <c r="G3" s="672"/>
+      <c r="H3" s="672"/>
+      <c r="I3" s="672"/>
+      <c r="J3" s="672"/>
+      <c r="K3" s="673" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="656" t="s">
+      <c r="L3" s="675" t="s">
         <v>310</v>
       </c>
       <c r="M3" s="20"/>
       <c r="N3" s="20"/>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" ht="25">
-      <c r="A4" s="646"/>
+      <c r="A4" s="665"/>
       <c r="B4" s="323"/>
-      <c r="C4" s="659"/>
+      <c r="C4" s="678"/>
       <c r="D4" s="387"/>
       <c r="E4" s="118" t="s">
         <v>595</v>
@@ -19855,8 +19876,8 @@
       <c r="J4" s="90" t="s">
         <v>113</v>
       </c>
-      <c r="K4" s="655"/>
-      <c r="L4" s="657"/>
+      <c r="K4" s="674"/>
+      <c r="L4" s="676"/>
       <c r="M4" s="20"/>
       <c r="N4" s="20"/>
     </row>
@@ -20967,80 +20988,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15">
-      <c r="A1" s="662" t="s">
+      <c r="A1" s="681" t="s">
         <v>329</v>
       </c>
-      <c r="B1" s="663"/>
-      <c r="C1" s="663"/>
-      <c r="D1" s="663"/>
-      <c r="E1" s="663"/>
-      <c r="F1" s="663"/>
-      <c r="G1" s="663"/>
-      <c r="H1" s="663"/>
-      <c r="I1" s="663"/>
-      <c r="J1" s="663"/>
-      <c r="K1" s="663"/>
-      <c r="L1" s="663"/>
-      <c r="M1" s="663"/>
-      <c r="N1" s="664"/>
+      <c r="B1" s="682"/>
+      <c r="C1" s="682"/>
+      <c r="D1" s="682"/>
+      <c r="E1" s="682"/>
+      <c r="F1" s="682"/>
+      <c r="G1" s="682"/>
+      <c r="H1" s="682"/>
+      <c r="I1" s="682"/>
+      <c r="J1" s="682"/>
+      <c r="K1" s="682"/>
+      <c r="L1" s="682"/>
+      <c r="M1" s="682"/>
+      <c r="N1" s="683"/>
       <c r="P1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="167" customFormat="1">
-      <c r="A2" s="665" t="s">
+      <c r="A2" s="684" t="s">
         <v>607</v>
       </c>
-      <c r="B2" s="666"/>
-      <c r="C2" s="666"/>
-      <c r="D2" s="666"/>
-      <c r="E2" s="666"/>
-      <c r="F2" s="666"/>
-      <c r="G2" s="666"/>
-      <c r="H2" s="666"/>
-      <c r="I2" s="666"/>
-      <c r="J2" s="666"/>
-      <c r="K2" s="666"/>
-      <c r="L2" s="666"/>
-      <c r="M2" s="666"/>
-      <c r="N2" s="667"/>
+      <c r="B2" s="685"/>
+      <c r="C2" s="685"/>
+      <c r="D2" s="685"/>
+      <c r="E2" s="685"/>
+      <c r="F2" s="685"/>
+      <c r="G2" s="685"/>
+      <c r="H2" s="685"/>
+      <c r="I2" s="685"/>
+      <c r="J2" s="685"/>
+      <c r="K2" s="685"/>
+      <c r="L2" s="685"/>
+      <c r="M2" s="685"/>
+      <c r="N2" s="686"/>
       <c r="O2" s="89"/>
       <c r="P2" s="89"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1">
-      <c r="A3" s="668"/>
+      <c r="A3" s="687"/>
       <c r="B3" s="336"/>
-      <c r="C3" s="672" t="s">
+      <c r="C3" s="691" t="s">
         <v>330</v>
       </c>
-      <c r="D3" s="660" t="s">
+      <c r="D3" s="679" t="s">
         <v>331</v>
       </c>
-      <c r="E3" s="672" t="s">
+      <c r="E3" s="691" t="s">
         <v>332</v>
       </c>
       <c r="F3" s="166"/>
-      <c r="G3" s="674" t="s">
+      <c r="G3" s="693" t="s">
         <v>605</v>
       </c>
-      <c r="H3" s="674"/>
-      <c r="I3" s="674"/>
-      <c r="J3" s="674"/>
-      <c r="K3" s="674"/>
-      <c r="L3" s="674"/>
-      <c r="M3" s="654" t="s">
+      <c r="H3" s="693"/>
+      <c r="I3" s="693"/>
+      <c r="J3" s="693"/>
+      <c r="K3" s="693"/>
+      <c r="L3" s="693"/>
+      <c r="M3" s="673" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="670" t="s">
+      <c r="N3" s="689" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="36">
-      <c r="A4" s="669"/>
+      <c r="A4" s="688"/>
       <c r="B4" s="337"/>
-      <c r="C4" s="673"/>
-      <c r="D4" s="661"/>
-      <c r="E4" s="673"/>
+      <c r="C4" s="692"/>
+      <c r="D4" s="680"/>
+      <c r="E4" s="692"/>
       <c r="F4" s="165"/>
       <c r="G4" s="118" t="s">
         <v>595</v>
@@ -21060,8 +21081,8 @@
       <c r="L4" s="90" t="s">
         <v>113</v>
       </c>
-      <c r="M4" s="655"/>
-      <c r="N4" s="671"/>
+      <c r="M4" s="674"/>
+      <c r="N4" s="690"/>
       <c r="O4" s="163"/>
       <c r="P4" s="163"/>
     </row>
@@ -22361,72 +22382,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15">
-      <c r="A1" s="662" t="s">
+      <c r="A1" s="681" t="s">
         <v>612</v>
       </c>
-      <c r="B1" s="663"/>
-      <c r="C1" s="663"/>
-      <c r="D1" s="663"/>
-      <c r="E1" s="663"/>
-      <c r="F1" s="663"/>
-      <c r="G1" s="663"/>
-      <c r="H1" s="663"/>
-      <c r="I1" s="663"/>
-      <c r="J1" s="663"/>
-      <c r="K1" s="663"/>
-      <c r="L1" s="663"/>
-      <c r="M1" s="664"/>
+      <c r="B1" s="682"/>
+      <c r="C1" s="682"/>
+      <c r="D1" s="682"/>
+      <c r="E1" s="682"/>
+      <c r="F1" s="682"/>
+      <c r="G1" s="682"/>
+      <c r="H1" s="682"/>
+      <c r="I1" s="682"/>
+      <c r="J1" s="682"/>
+      <c r="K1" s="682"/>
+      <c r="L1" s="682"/>
+      <c r="M1" s="683"/>
       <c r="O1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="167" customFormat="1">
-      <c r="A2" s="675" t="s">
+      <c r="A2" s="694" t="s">
         <v>623</v>
       </c>
-      <c r="B2" s="676"/>
-      <c r="C2" s="676"/>
-      <c r="D2" s="676"/>
-      <c r="E2" s="676"/>
-      <c r="F2" s="676"/>
-      <c r="G2" s="676"/>
-      <c r="H2" s="676"/>
-      <c r="I2" s="676"/>
-      <c r="J2" s="676"/>
-      <c r="K2" s="676"/>
-      <c r="L2" s="676"/>
-      <c r="M2" s="677"/>
+      <c r="B2" s="695"/>
+      <c r="C2" s="695"/>
+      <c r="D2" s="695"/>
+      <c r="E2" s="695"/>
+      <c r="F2" s="695"/>
+      <c r="G2" s="695"/>
+      <c r="H2" s="695"/>
+      <c r="I2" s="695"/>
+      <c r="J2" s="695"/>
+      <c r="K2" s="695"/>
+      <c r="L2" s="695"/>
+      <c r="M2" s="696"/>
       <c r="N2" s="89"/>
       <c r="O2" s="89"/>
     </row>
     <row r="3" spans="1:15" ht="12.75" customHeight="1">
-      <c r="A3" s="668"/>
+      <c r="A3" s="687"/>
       <c r="B3" s="336"/>
-      <c r="C3" s="672" t="s">
+      <c r="C3" s="691" t="s">
         <v>609</v>
       </c>
-      <c r="D3" s="672" t="s">
+      <c r="D3" s="691" t="s">
         <v>610</v>
       </c>
       <c r="E3" s="166"/>
       <c r="F3" s="166"/>
-      <c r="G3" s="616" t="s">
+      <c r="G3" s="635" t="s">
         <v>624</v>
       </c>
-      <c r="H3" s="616"/>
-      <c r="I3" s="616"/>
-      <c r="J3" s="616"/>
-      <c r="K3" s="616"/>
-      <c r="L3" s="616"/>
-      <c r="M3" s="678" t="s">
+      <c r="H3" s="635"/>
+      <c r="I3" s="635"/>
+      <c r="J3" s="635"/>
+      <c r="K3" s="635"/>
+      <c r="L3" s="635"/>
+      <c r="M3" s="697" t="s">
         <v>613</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="24">
-      <c r="A4" s="669"/>
+      <c r="A4" s="688"/>
       <c r="B4" s="337"/>
-      <c r="C4" s="673"/>
-      <c r="D4" s="673"/>
+      <c r="C4" s="692"/>
+      <c r="D4" s="692"/>
       <c r="E4" s="165"/>
       <c r="F4" s="165"/>
       <c r="G4" s="102" t="s">
@@ -22447,7 +22468,7 @@
       <c r="L4" s="102" t="s">
         <v>113</v>
       </c>
-      <c r="M4" s="679"/>
+      <c r="M4" s="698"/>
       <c r="N4" s="163"/>
       <c r="O4" s="163"/>
     </row>
@@ -23686,46 +23707,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>629</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="611"/>
     </row>
     <row r="2" spans="1:5" s="31" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A2" s="683" t="s">
+      <c r="A2" s="702" t="s">
         <v>632</v>
       </c>
-      <c r="B2" s="684"/>
-      <c r="C2" s="684"/>
-      <c r="D2" s="684"/>
-      <c r="E2" s="685"/>
+      <c r="B2" s="703"/>
+      <c r="C2" s="703"/>
+      <c r="D2" s="703"/>
+      <c r="E2" s="704"/>
     </row>
     <row r="3" spans="1:5" s="31" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A3" s="686"/>
-      <c r="B3" s="688" t="s">
+      <c r="A3" s="705"/>
+      <c r="B3" s="707" t="s">
         <v>630</v>
       </c>
-      <c r="C3" s="688"/>
-      <c r="D3" s="689" t="s">
+      <c r="C3" s="707"/>
+      <c r="D3" s="708" t="s">
         <v>631</v>
       </c>
-      <c r="E3" s="690" t="s">
+      <c r="E3" s="709" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="31" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A4" s="687"/>
+      <c r="A4" s="706"/>
       <c r="B4" s="84" t="s">
         <v>347</v>
       </c>
       <c r="C4" s="84" t="s">
         <v>348</v>
       </c>
-      <c r="D4" s="581"/>
-      <c r="E4" s="691"/>
+      <c r="D4" s="600"/>
+      <c r="E4" s="710"/>
     </row>
     <row r="5" spans="1:5" ht="11.25" customHeight="1">
       <c r="A5" s="168"/>
@@ -24429,13 +24450,13 @@
       <c r="E47" s="182"/>
     </row>
     <row r="48" spans="1:21" ht="22.5" customHeight="1">
-      <c r="A48" s="680" t="s">
+      <c r="A48" s="699" t="s">
         <v>351</v>
       </c>
-      <c r="B48" s="681"/>
-      <c r="C48" s="681"/>
-      <c r="D48" s="681"/>
-      <c r="E48" s="682"/>
+      <c r="B48" s="700"/>
+      <c r="C48" s="700"/>
+      <c r="D48" s="700"/>
+      <c r="E48" s="701"/>
     </row>
     <row r="49" spans="2:4">
       <c r="B49" s="183"/>
@@ -24599,7 +24620,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{305B2D60-C2CA-F14D-A8B1-1BCB1D99F6E3}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="95.83203125" customWidth="1"/>
@@ -24619,6 +24640,31 @@
       <c r="A3" s="554" t="s">
         <v>770</v>
       </c>
+    </row>
+    <row r="4" spans="1:1" ht="395">
+      <ns0:c xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="A4" s="554" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"># Extra table: FIES ----------------------------------------------------
+extra_tables_dict &lt;- list(
+  "4.1" = "tb_41"
+)
+tables_extra &lt;- names(extra_tables_dict)
+# Preserve prepared datasets in case the FIES script overwrites them.
+hh_before_fies &lt;- hh
+hl_before_fies &lt;- hl
+# Senegal FIES script: country code SEN, Wave 1, Table 4.1.
+source(
+  file.path(path_fies, "SEN MICSPlus Wave1 - Table 4.1_Script.R"),
+  local = TRUE
+)
+# If the script returns res.df rather than tb_41,
+# insert the conversion of its results into tb_41 here.
+stopifnot(exists("tb_41", inherits = FALSE))
+hh &lt;- hh_before_fies
+hl &lt;- hl_before_fies
+</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
@@ -24655,82 +24701,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>352</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="696"/>
-      <c r="E1" s="696"/>
-      <c r="F1" s="696"/>
-      <c r="G1" s="696"/>
-      <c r="H1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="562"/>
+      <c r="E1" s="562"/>
+      <c r="F1" s="562"/>
+      <c r="G1" s="562"/>
+      <c r="H1" s="563"/>
       <c r="I1" s="186"/>
       <c r="J1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="12" customHeight="1">
-      <c r="A2" s="698" t="s">
+      <c r="A2" s="711" t="s">
         <v>353</v>
       </c>
-      <c r="B2" s="699"/>
-      <c r="C2" s="699"/>
-      <c r="D2" s="699"/>
-      <c r="E2" s="699"/>
-      <c r="F2" s="699"/>
-      <c r="G2" s="699"/>
-      <c r="H2" s="700"/>
+      <c r="B2" s="712"/>
+      <c r="C2" s="712"/>
+      <c r="D2" s="712"/>
+      <c r="E2" s="712"/>
+      <c r="F2" s="712"/>
+      <c r="G2" s="712"/>
+      <c r="H2" s="713"/>
       <c r="I2" s="188"/>
       <c r="K2" s="190"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="701"/>
+      <c r="A3" s="714"/>
       <c r="B3" s="376"/>
-      <c r="C3" s="704" t="s">
+      <c r="C3" s="570" t="s">
         <v>637</v>
       </c>
-      <c r="D3" s="704"/>
-      <c r="E3" s="704"/>
-      <c r="F3" s="704"/>
-      <c r="G3" s="705"/>
-      <c r="H3" s="706" t="s">
+      <c r="D3" s="570"/>
+      <c r="E3" s="570"/>
+      <c r="F3" s="570"/>
+      <c r="G3" s="717"/>
+      <c r="H3" s="572" t="s">
         <v>354</v>
       </c>
       <c r="I3" s="192"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="702"/>
+      <c r="A4" s="715"/>
       <c r="B4" s="377"/>
-      <c r="C4" s="709" t="s">
+      <c r="C4" s="719" t="s">
         <v>355</v>
       </c>
-      <c r="D4" s="709" t="s">
+      <c r="D4" s="719" t="s">
         <v>356</v>
       </c>
-      <c r="E4" s="711" t="s">
+      <c r="E4" s="721" t="s">
         <v>357</v>
       </c>
-      <c r="F4" s="711"/>
-      <c r="G4" s="709" t="s">
+      <c r="F4" s="721"/>
+      <c r="G4" s="719" t="s">
         <v>358</v>
       </c>
-      <c r="H4" s="707"/>
+      <c r="H4" s="573"/>
       <c r="I4" s="192"/>
     </row>
     <row r="5" spans="1:11" ht="14">
-      <c r="A5" s="703"/>
+      <c r="A5" s="716"/>
       <c r="B5" s="378"/>
-      <c r="C5" s="710"/>
-      <c r="D5" s="710"/>
+      <c r="C5" s="720"/>
+      <c r="D5" s="720"/>
       <c r="E5" s="193" t="s">
         <v>359</v>
       </c>
       <c r="F5" s="193" t="s">
         <v>360</v>
       </c>
-      <c r="G5" s="710"/>
-      <c r="H5" s="708"/>
+      <c r="G5" s="720"/>
+      <c r="H5" s="718"/>
       <c r="I5" s="194"/>
     </row>
     <row r="6" spans="1:11" ht="60">
@@ -25844,16 +25890,16 @@
       <c r="I54" s="448"/>
     </row>
     <row r="55" spans="1:9">
-      <c r="A55" s="692" t="s">
+      <c r="A55" s="564" t="s">
         <v>368</v>
       </c>
-      <c r="B55" s="693"/>
-      <c r="C55" s="693"/>
-      <c r="D55" s="693"/>
-      <c r="E55" s="693"/>
-      <c r="F55" s="693"/>
-      <c r="G55" s="693"/>
-      <c r="H55" s="694"/>
+      <c r="B55" s="565"/>
+      <c r="C55" s="565"/>
+      <c r="D55" s="565"/>
+      <c r="E55" s="565"/>
+      <c r="F55" s="565"/>
+      <c r="G55" s="565"/>
+      <c r="H55" s="566"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -25899,24 +25945,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="563"/>
       <c r="E1" s="186"/>
       <c r="F1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="23.75" customHeight="1">
-      <c r="A2" s="698" t="s">
+      <c r="A2" s="711" t="s">
         <v>370</v>
       </c>
-      <c r="B2" s="699"/>
-      <c r="C2" s="699"/>
-      <c r="D2" s="700"/>
+      <c r="B2" s="712"/>
+      <c r="C2" s="712"/>
+      <c r="D2" s="713"/>
       <c r="E2" s="201"/>
     </row>
     <row r="3" spans="1:6" ht="36">
@@ -27050,12 +27096,12 @@
       <c r="E53" s="454"/>
     </row>
     <row r="54" spans="1:23" s="210" customFormat="1" ht="36.5" customHeight="1">
-      <c r="A54" s="712" t="s">
+      <c r="A54" s="722" t="s">
         <v>375</v>
       </c>
-      <c r="B54" s="713"/>
-      <c r="C54" s="713"/>
-      <c r="D54" s="714"/>
+      <c r="B54" s="723"/>
+      <c r="C54" s="723"/>
+      <c r="D54" s="724"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -27102,73 +27148,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>652</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="696"/>
-      <c r="E1" s="696"/>
-      <c r="F1" s="696"/>
-      <c r="G1" s="696"/>
-      <c r="H1" s="696"/>
-      <c r="I1" s="696"/>
-      <c r="J1" s="696"/>
-      <c r="K1" s="696"/>
-      <c r="L1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="562"/>
+      <c r="E1" s="562"/>
+      <c r="F1" s="562"/>
+      <c r="G1" s="562"/>
+      <c r="H1" s="562"/>
+      <c r="I1" s="562"/>
+      <c r="J1" s="562"/>
+      <c r="K1" s="562"/>
+      <c r="L1" s="563"/>
       <c r="M1" s="186"/>
       <c r="N1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="692" t="s">
+      <c r="A2" s="564" t="s">
         <v>657</v>
       </c>
-      <c r="B2" s="693"/>
-      <c r="C2" s="693"/>
-      <c r="D2" s="693"/>
-      <c r="E2" s="693"/>
-      <c r="F2" s="693"/>
-      <c r="G2" s="693"/>
-      <c r="H2" s="693"/>
-      <c r="I2" s="693"/>
-      <c r="J2" s="693"/>
-      <c r="K2" s="693"/>
-      <c r="L2" s="694"/>
+      <c r="B2" s="565"/>
+      <c r="C2" s="565"/>
+      <c r="D2" s="565"/>
+      <c r="E2" s="565"/>
+      <c r="F2" s="565"/>
+      <c r="G2" s="565"/>
+      <c r="H2" s="565"/>
+      <c r="I2" s="565"/>
+      <c r="J2" s="565"/>
+      <c r="K2" s="565"/>
+      <c r="L2" s="566"/>
       <c r="M2" s="211"/>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="715"/>
+      <c r="A3" s="567"/>
       <c r="B3" s="212"/>
-      <c r="C3" s="717" t="s">
+      <c r="C3" s="559" t="s">
         <v>653</v>
       </c>
-      <c r="D3" s="717" t="s">
+      <c r="D3" s="559" t="s">
         <v>464</v>
       </c>
       <c r="E3" s="212"/>
-      <c r="F3" s="704" t="s">
+      <c r="F3" s="570" t="s">
         <v>489</v>
       </c>
-      <c r="G3" s="704"/>
-      <c r="H3" s="717" t="s">
+      <c r="G3" s="570"/>
+      <c r="H3" s="559" t="s">
         <v>465</v>
       </c>
-      <c r="J3" s="704" t="s">
+      <c r="J3" s="570" t="s">
         <v>489</v>
       </c>
-      <c r="K3" s="704"/>
-      <c r="L3" s="706" t="s">
+      <c r="K3" s="570"/>
+      <c r="L3" s="572" t="s">
         <v>466</v>
       </c>
       <c r="M3" s="205"/>
     </row>
     <row r="4" spans="1:14" ht="24">
-      <c r="A4" s="716"/>
+      <c r="A4" s="569"/>
       <c r="B4" s="213"/>
-      <c r="C4" s="718"/>
-      <c r="D4" s="718"/>
+      <c r="C4" s="560"/>
+      <c r="D4" s="560"/>
       <c r="E4" s="213"/>
       <c r="F4" s="213" t="s">
         <v>467</v>
@@ -27176,14 +27222,14 @@
       <c r="G4" s="213" t="s">
         <v>468</v>
       </c>
-      <c r="H4" s="718"/>
+      <c r="H4" s="560"/>
       <c r="J4" s="213" t="s">
         <v>469</v>
       </c>
       <c r="K4" s="213" t="s">
         <v>470</v>
       </c>
-      <c r="L4" s="719"/>
+      <c r="L4" s="574"/>
       <c r="M4" s="205"/>
     </row>
     <row r="5" spans="1:14" ht="86" customHeight="1">
@@ -28394,54 +28440,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>766</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="696"/>
-      <c r="E1" s="696"/>
-      <c r="F1" s="696"/>
-      <c r="G1" s="696"/>
-      <c r="H1" s="696"/>
-      <c r="I1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="562"/>
+      <c r="E1" s="562"/>
+      <c r="F1" s="562"/>
+      <c r="G1" s="562"/>
+      <c r="H1" s="562"/>
+      <c r="I1" s="563"/>
       <c r="K1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
-      <c r="A2" s="692" t="s">
+      <c r="A2" s="564" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="693"/>
-      <c r="C2" s="693"/>
-      <c r="D2" s="693"/>
-      <c r="E2" s="693"/>
-      <c r="F2" s="693"/>
-      <c r="G2" s="693"/>
-      <c r="H2" s="693"/>
-      <c r="I2" s="694"/>
+      <c r="B2" s="565"/>
+      <c r="C2" s="565"/>
+      <c r="D2" s="565"/>
+      <c r="E2" s="565"/>
+      <c r="F2" s="565"/>
+      <c r="G2" s="565"/>
+      <c r="H2" s="565"/>
+      <c r="I2" s="566"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="715"/>
+      <c r="A3" s="567"/>
       <c r="B3" s="212"/>
-      <c r="C3" s="704" t="s">
+      <c r="C3" s="570" t="s">
         <v>489</v>
       </c>
-      <c r="D3" s="704"/>
-      <c r="E3" s="717" t="s">
+      <c r="D3" s="570"/>
+      <c r="E3" s="559" t="s">
         <v>464</v>
       </c>
-      <c r="G3" s="704" t="s">
+      <c r="G3" s="570" t="s">
         <v>489</v>
       </c>
-      <c r="H3" s="704"/>
-      <c r="I3" s="706" t="s">
+      <c r="H3" s="570"/>
+      <c r="I3" s="572" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="24">
-      <c r="A4" s="716"/>
+      <c r="A4" s="569"/>
       <c r="B4" s="213"/>
       <c r="C4" s="213" t="s">
         <v>475</v>
@@ -28449,14 +28495,14 @@
       <c r="D4" s="213" t="s">
         <v>476</v>
       </c>
-      <c r="E4" s="718"/>
+      <c r="E4" s="560"/>
       <c r="G4" s="213" t="s">
         <v>475</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>476</v>
       </c>
-      <c r="I4" s="719"/>
+      <c r="I4" s="574"/>
       <c r="J4" s="208"/>
     </row>
     <row r="5" spans="1:13" ht="120">
@@ -29496,17 +29542,17 @@
       <c r="J47" s="472"/>
     </row>
     <row r="48" spans="1:27" ht="12" customHeight="1">
-      <c r="A48" s="692" t="s">
+      <c r="A48" s="564" t="s">
         <v>477</v>
       </c>
-      <c r="B48" s="693"/>
-      <c r="C48" s="693"/>
-      <c r="D48" s="693"/>
-      <c r="E48" s="693"/>
-      <c r="F48" s="693"/>
-      <c r="G48" s="693"/>
-      <c r="H48" s="693"/>
-      <c r="I48" s="694"/>
+      <c r="B48" s="565"/>
+      <c r="C48" s="565"/>
+      <c r="D48" s="565"/>
+      <c r="E48" s="565"/>
+      <c r="F48" s="565"/>
+      <c r="G48" s="565"/>
+      <c r="H48" s="565"/>
+      <c r="I48" s="566"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -29870,55 +29916,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>767</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="696"/>
-      <c r="E1" s="696"/>
-      <c r="F1" s="696"/>
-      <c r="G1" s="696"/>
-      <c r="H1" s="696"/>
-      <c r="I1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="562"/>
+      <c r="E1" s="562"/>
+      <c r="F1" s="562"/>
+      <c r="G1" s="562"/>
+      <c r="H1" s="562"/>
+      <c r="I1" s="563"/>
       <c r="K1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="692" t="s">
+      <c r="A2" s="564" t="s">
         <v>659</v>
       </c>
-      <c r="B2" s="693"/>
-      <c r="C2" s="693"/>
-      <c r="D2" s="693"/>
-      <c r="E2" s="693"/>
-      <c r="F2" s="693"/>
-      <c r="G2" s="693"/>
-      <c r="H2" s="693"/>
-      <c r="I2" s="694"/>
+      <c r="B2" s="565"/>
+      <c r="C2" s="565"/>
+      <c r="D2" s="565"/>
+      <c r="E2" s="565"/>
+      <c r="F2" s="565"/>
+      <c r="G2" s="565"/>
+      <c r="H2" s="565"/>
+      <c r="I2" s="566"/>
     </row>
     <row r="3" spans="1:13" ht="21.5" customHeight="1">
-      <c r="A3" s="715"/>
+      <c r="A3" s="567"/>
       <c r="B3" s="212"/>
-      <c r="C3" s="704" t="s">
+      <c r="C3" s="570" t="s">
         <v>478</v>
       </c>
-      <c r="D3" s="704"/>
+      <c r="D3" s="570"/>
       <c r="E3" s="212"/>
-      <c r="F3" s="704" t="s">
+      <c r="F3" s="570" t="s">
         <v>658</v>
       </c>
-      <c r="G3" s="704"/>
-      <c r="H3" s="717" t="s">
+      <c r="G3" s="570"/>
+      <c r="H3" s="559" t="s">
         <v>479</v>
       </c>
-      <c r="I3" s="706" t="s">
+      <c r="I3" s="572" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="23.5" customHeight="1">
-      <c r="A4" s="716"/>
+      <c r="A4" s="569"/>
       <c r="B4" s="213"/>
       <c r="C4" s="213" t="s">
         <v>481</v>
@@ -29933,8 +29979,8 @@
       <c r="G4" s="213" t="s">
         <v>482</v>
       </c>
-      <c r="H4" s="718"/>
-      <c r="I4" s="719"/>
+      <c r="H4" s="560"/>
+      <c r="I4" s="574"/>
     </row>
     <row r="5" spans="1:13" ht="317">
       <c r="A5" s="195"/>
@@ -31023,17 +31069,17 @@
       <c r="J51" s="472"/>
     </row>
     <row r="52" spans="1:10">
-      <c r="A52" s="720" t="s">
+      <c r="A52" s="556" t="s">
         <v>487</v>
       </c>
-      <c r="B52" s="721"/>
-      <c r="C52" s="721"/>
-      <c r="D52" s="721"/>
-      <c r="E52" s="721"/>
-      <c r="F52" s="721"/>
-      <c r="G52" s="721"/>
-      <c r="H52" s="721"/>
-      <c r="I52" s="722"/>
+      <c r="B52" s="557"/>
+      <c r="C52" s="557"/>
+      <c r="D52" s="557"/>
+      <c r="E52" s="557"/>
+      <c r="F52" s="557"/>
+      <c r="G52" s="557"/>
+      <c r="H52" s="557"/>
+      <c r="I52" s="558"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -31088,131 +31134,131 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="187" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="695" t="s">
+      <c r="A1" s="561" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="696"/>
-      <c r="C1" s="696"/>
-      <c r="D1" s="696"/>
-      <c r="E1" s="696"/>
-      <c r="F1" s="696"/>
-      <c r="G1" s="696"/>
-      <c r="H1" s="696"/>
-      <c r="I1" s="696"/>
-      <c r="J1" s="696"/>
-      <c r="K1" s="696"/>
-      <c r="L1" s="696"/>
-      <c r="M1" s="696"/>
-      <c r="N1" s="696"/>
-      <c r="O1" s="696"/>
-      <c r="P1" s="697"/>
+      <c r="B1" s="562"/>
+      <c r="C1" s="562"/>
+      <c r="D1" s="562"/>
+      <c r="E1" s="562"/>
+      <c r="F1" s="562"/>
+      <c r="G1" s="562"/>
+      <c r="H1" s="562"/>
+      <c r="I1" s="562"/>
+      <c r="J1" s="562"/>
+      <c r="K1" s="562"/>
+      <c r="L1" s="562"/>
+      <c r="M1" s="562"/>
+      <c r="N1" s="562"/>
+      <c r="O1" s="562"/>
+      <c r="P1" s="563"/>
       <c r="R1" s="91" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
-      <c r="A2" s="692" t="s">
+      <c r="A2" s="564" t="s">
         <v>488</v>
       </c>
-      <c r="B2" s="693"/>
-      <c r="C2" s="693"/>
-      <c r="D2" s="693"/>
-      <c r="E2" s="693"/>
-      <c r="F2" s="693"/>
-      <c r="G2" s="693"/>
-      <c r="H2" s="693"/>
-      <c r="I2" s="693"/>
-      <c r="J2" s="693"/>
-      <c r="K2" s="693"/>
-      <c r="L2" s="693"/>
-      <c r="M2" s="693"/>
-      <c r="N2" s="693"/>
-      <c r="O2" s="693"/>
-      <c r="P2" s="694"/>
+      <c r="B2" s="565"/>
+      <c r="C2" s="565"/>
+      <c r="D2" s="565"/>
+      <c r="E2" s="565"/>
+      <c r="F2" s="565"/>
+      <c r="G2" s="565"/>
+      <c r="H2" s="565"/>
+      <c r="I2" s="565"/>
+      <c r="J2" s="565"/>
+      <c r="K2" s="565"/>
+      <c r="L2" s="565"/>
+      <c r="M2" s="565"/>
+      <c r="N2" s="565"/>
+      <c r="O2" s="565"/>
+      <c r="P2" s="566"/>
     </row>
     <row r="3" spans="1:18" ht="12" customHeight="1">
-      <c r="A3" s="715"/>
+      <c r="A3" s="567"/>
       <c r="B3" s="212"/>
-      <c r="C3" s="704" t="s">
+      <c r="C3" s="570" t="s">
         <v>489</v>
       </c>
-      <c r="D3" s="704"/>
-      <c r="E3" s="717"/>
-      <c r="F3" s="704" t="s">
+      <c r="D3" s="570"/>
+      <c r="E3" s="559"/>
+      <c r="F3" s="570" t="s">
         <v>490</v>
       </c>
-      <c r="G3" s="704"/>
-      <c r="H3" s="704"/>
-      <c r="I3" s="704"/>
-      <c r="J3" s="704"/>
-      <c r="K3" s="704"/>
-      <c r="L3" s="704"/>
-      <c r="M3" s="704"/>
-      <c r="N3" s="704"/>
-      <c r="O3" s="717" t="s">
+      <c r="G3" s="570"/>
+      <c r="H3" s="570"/>
+      <c r="I3" s="570"/>
+      <c r="J3" s="570"/>
+      <c r="K3" s="570"/>
+      <c r="L3" s="570"/>
+      <c r="M3" s="570"/>
+      <c r="N3" s="570"/>
+      <c r="O3" s="559" t="s">
         <v>491</v>
       </c>
-      <c r="P3" s="706" t="s">
+      <c r="P3" s="572" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="22.5" customHeight="1">
-      <c r="A4" s="723"/>
+      <c r="A4" s="568"/>
       <c r="B4" s="192"/>
-      <c r="C4" s="724" t="s">
+      <c r="C4" s="571" t="s">
         <v>492</v>
       </c>
-      <c r="D4" s="724" t="s">
+      <c r="D4" s="571" t="s">
         <v>493</v>
       </c>
-      <c r="E4" s="724"/>
-      <c r="F4" s="717" t="s">
+      <c r="E4" s="571"/>
+      <c r="F4" s="559" t="s">
         <v>494</v>
       </c>
-      <c r="G4" s="717" t="s">
+      <c r="G4" s="559" t="s">
         <v>495</v>
       </c>
-      <c r="H4" s="717" t="s">
+      <c r="H4" s="559" t="s">
         <v>496</v>
       </c>
-      <c r="I4" s="717" t="s">
+      <c r="I4" s="559" t="s">
         <v>497</v>
       </c>
-      <c r="J4" s="717" t="s">
+      <c r="J4" s="559" t="s">
         <v>498</v>
       </c>
-      <c r="K4" s="717" t="s">
+      <c r="K4" s="559" t="s">
         <v>499</v>
       </c>
-      <c r="L4" s="717" t="s">
+      <c r="L4" s="559" t="s">
         <v>500</v>
       </c>
-      <c r="M4" s="717" t="s">
+      <c r="M4" s="559" t="s">
         <v>501</v>
       </c>
-      <c r="N4" s="717" t="s">
+      <c r="N4" s="559" t="s">
         <v>502</v>
       </c>
-      <c r="O4" s="724"/>
-      <c r="P4" s="707"/>
+      <c r="O4" s="571"/>
+      <c r="P4" s="573"/>
     </row>
     <row r="5" spans="1:18">
-      <c r="A5" s="716"/>
+      <c r="A5" s="569"/>
       <c r="B5" s="213"/>
-      <c r="C5" s="718"/>
-      <c r="D5" s="718"/>
-      <c r="E5" s="718"/>
-      <c r="F5" s="718"/>
-      <c r="G5" s="718"/>
-      <c r="H5" s="718"/>
-      <c r="I5" s="718"/>
-      <c r="J5" s="718"/>
-      <c r="K5" s="718"/>
-      <c r="L5" s="718"/>
-      <c r="M5" s="718"/>
-      <c r="N5" s="718"/>
-      <c r="O5" s="718"/>
-      <c r="P5" s="719"/>
+      <c r="C5" s="560"/>
+      <c r="D5" s="560"/>
+      <c r="E5" s="560"/>
+      <c r="F5" s="560"/>
+      <c r="G5" s="560"/>
+      <c r="H5" s="560"/>
+      <c r="I5" s="560"/>
+      <c r="J5" s="560"/>
+      <c r="K5" s="560"/>
+      <c r="L5" s="560"/>
+      <c r="M5" s="560"/>
+      <c r="N5" s="560"/>
+      <c r="O5" s="560"/>
+      <c r="P5" s="574"/>
     </row>
     <row r="6" spans="1:18" ht="408" customHeight="1">
       <c r="A6" s="195"/>
@@ -32503,33 +32549,27 @@
       <c r="Q52" s="472"/>
     </row>
     <row r="53" spans="1:18" ht="12" customHeight="1">
-      <c r="A53" s="720" t="s">
+      <c r="A53" s="556" t="s">
         <v>487</v>
       </c>
-      <c r="B53" s="721"/>
-      <c r="C53" s="721"/>
-      <c r="D53" s="721"/>
-      <c r="E53" s="721"/>
-      <c r="F53" s="721"/>
-      <c r="G53" s="721"/>
-      <c r="H53" s="721"/>
-      <c r="I53" s="721"/>
-      <c r="J53" s="721"/>
-      <c r="K53" s="721"/>
-      <c r="L53" s="721"/>
-      <c r="M53" s="721"/>
-      <c r="N53" s="721"/>
-      <c r="O53" s="721"/>
-      <c r="P53" s="722"/>
+      <c r="B53" s="557"/>
+      <c r="C53" s="557"/>
+      <c r="D53" s="557"/>
+      <c r="E53" s="557"/>
+      <c r="F53" s="557"/>
+      <c r="G53" s="557"/>
+      <c r="H53" s="557"/>
+      <c r="I53" s="557"/>
+      <c r="J53" s="557"/>
+      <c r="K53" s="557"/>
+      <c r="L53" s="557"/>
+      <c r="M53" s="557"/>
+      <c r="N53" s="557"/>
+      <c r="O53" s="557"/>
+      <c r="P53" s="558"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A53:P53"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A3:A5"/>
@@ -32544,6 +32584,12 @@
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="N4:N5"/>
+    <mergeCell ref="A53:P53"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
   </mergeCells>
   <phoneticPr fontId="31" type="noConversion"/>
   <hyperlinks>
@@ -32592,32 +32638,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>708</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="591"/>
-      <c r="K1" s="591"/>
-      <c r="L1" s="591"/>
-      <c r="M1" s="591"/>
-      <c r="N1" s="591"/>
-      <c r="O1" s="591"/>
-      <c r="P1" s="591"/>
-      <c r="Q1" s="591"/>
-      <c r="R1" s="591"/>
-      <c r="S1" s="591"/>
-      <c r="T1" s="591"/>
-      <c r="U1" s="591"/>
-      <c r="V1" s="591"/>
-      <c r="W1" s="591"/>
-      <c r="X1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="610"/>
+      <c r="K1" s="610"/>
+      <c r="L1" s="610"/>
+      <c r="M1" s="610"/>
+      <c r="N1" s="610"/>
+      <c r="O1" s="610"/>
+      <c r="P1" s="610"/>
+      <c r="Q1" s="610"/>
+      <c r="R1" s="610"/>
+      <c r="S1" s="610"/>
+      <c r="T1" s="610"/>
+      <c r="U1" s="610"/>
+      <c r="V1" s="610"/>
+      <c r="W1" s="610"/>
+      <c r="X1" s="611"/>
       <c r="Y1" s="89"/>
       <c r="Z1" s="478" t="s">
         <v>7</v>
@@ -32699,11 +32745,11 @@
       <c r="I4" s="732"/>
       <c r="J4" s="732"/>
       <c r="K4" s="732"/>
-      <c r="L4" s="689"/>
-      <c r="M4" s="689"/>
-      <c r="N4" s="689"/>
-      <c r="O4" s="689"/>
-      <c r="P4" s="689"/>
+      <c r="L4" s="708"/>
+      <c r="M4" s="708"/>
+      <c r="N4" s="708"/>
+      <c r="O4" s="708"/>
+      <c r="P4" s="708"/>
       <c r="Q4" s="734"/>
       <c r="R4" s="731" t="s">
         <v>379</v>
@@ -32711,9 +32757,9 @@
       <c r="S4" s="731"/>
       <c r="T4" s="731"/>
       <c r="U4" s="731"/>
-      <c r="V4" s="581"/>
-      <c r="W4" s="581"/>
-      <c r="X4" s="691"/>
+      <c r="V4" s="600"/>
+      <c r="W4" s="600"/>
+      <c r="X4" s="710"/>
     </row>
     <row r="5" spans="1:26" ht="12" customHeight="1">
       <c r="A5" s="729"/>
@@ -32723,47 +32769,47 @@
       </c>
       <c r="D5" s="735"/>
       <c r="E5" s="735"/>
-      <c r="F5" s="581"/>
-      <c r="G5" s="689" t="s">
+      <c r="F5" s="600"/>
+      <c r="G5" s="708" t="s">
         <v>381</v>
       </c>
-      <c r="H5" s="689" t="s">
+      <c r="H5" s="708" t="s">
         <v>382</v>
       </c>
-      <c r="I5" s="689" t="s">
+      <c r="I5" s="708" t="s">
         <v>383</v>
       </c>
-      <c r="J5" s="689" t="s">
+      <c r="J5" s="708" t="s">
         <v>384</v>
       </c>
-      <c r="K5" s="689" t="s">
+      <c r="K5" s="708" t="s">
         <v>385</v>
       </c>
       <c r="L5" s="117"/>
       <c r="M5" s="117"/>
-      <c r="N5" s="689" t="s">
+      <c r="N5" s="708" t="s">
         <v>703</v>
       </c>
       <c r="O5" s="117"/>
-      <c r="P5" s="689" t="s">
+      <c r="P5" s="708" t="s">
         <v>699</v>
       </c>
-      <c r="Q5" s="582"/>
-      <c r="R5" s="689" t="s">
+      <c r="Q5" s="601"/>
+      <c r="R5" s="708" t="s">
         <v>388</v>
       </c>
-      <c r="S5" s="689" t="s">
+      <c r="S5" s="708" t="s">
         <v>389</v>
       </c>
-      <c r="T5" s="689" t="s">
+      <c r="T5" s="708" t="s">
         <v>390</v>
       </c>
-      <c r="U5" s="689" t="s">
+      <c r="U5" s="708" t="s">
         <v>59</v>
       </c>
-      <c r="V5" s="581"/>
-      <c r="W5" s="581"/>
-      <c r="X5" s="691"/>
+      <c r="V5" s="600"/>
+      <c r="W5" s="600"/>
+      <c r="X5" s="710"/>
     </row>
     <row r="6" spans="1:26" ht="24">
       <c r="A6" s="730"/>
@@ -32780,30 +32826,30 @@
       <c r="F6" s="84" t="s">
         <v>394</v>
       </c>
-      <c r="G6" s="581"/>
-      <c r="H6" s="581"/>
-      <c r="I6" s="581"/>
-      <c r="J6" s="581"/>
-      <c r="K6" s="581"/>
+      <c r="G6" s="600"/>
+      <c r="H6" s="600"/>
+      <c r="I6" s="600"/>
+      <c r="J6" s="600"/>
+      <c r="K6" s="600"/>
       <c r="L6" s="84" t="s">
         <v>395</v>
       </c>
       <c r="M6" s="84" t="s">
         <v>386</v>
       </c>
-      <c r="N6" s="581"/>
+      <c r="N6" s="600"/>
       <c r="O6" s="84" t="s">
         <v>387</v>
       </c>
-      <c r="P6" s="581"/>
+      <c r="P6" s="600"/>
       <c r="Q6" s="735"/>
-      <c r="R6" s="581"/>
-      <c r="S6" s="581"/>
-      <c r="T6" s="581"/>
-      <c r="U6" s="581"/>
-      <c r="V6" s="581"/>
-      <c r="W6" s="581"/>
-      <c r="X6" s="691"/>
+      <c r="R6" s="600"/>
+      <c r="S6" s="600"/>
+      <c r="T6" s="600"/>
+      <c r="U6" s="600"/>
+      <c r="V6" s="600"/>
+      <c r="W6" s="600"/>
+      <c r="X6" s="710"/>
     </row>
     <row r="7" spans="1:26" ht="48">
       <c r="A7" s="50"/>
@@ -34068,12 +34114,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="S5:S6"/>
-    <mergeCell ref="T5:T6"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="A2:X2"/>
     <mergeCell ref="A3:A6"/>
@@ -34090,6 +34130,12 @@
     <mergeCell ref="H5:H6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="J5:J6"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="S5:S6"/>
+    <mergeCell ref="T5:T6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Z1" location="IDX!A1" display="IDX" xr:uid="{0F3E965F-DE71-43B7-89DA-A55C616FFDE1}"/>
@@ -34130,22 +34176,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>709</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="591"/>
-      <c r="K1" s="591"/>
-      <c r="L1" s="591"/>
-      <c r="M1" s="591"/>
-      <c r="N1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="610"/>
+      <c r="K1" s="610"/>
+      <c r="L1" s="610"/>
+      <c r="M1" s="610"/>
+      <c r="N1" s="611"/>
       <c r="O1" s="89"/>
       <c r="P1" s="478" t="s">
         <v>7</v>
@@ -34183,7 +34229,7 @@
       <c r="I3" s="731"/>
       <c r="J3" s="731"/>
       <c r="K3" s="731"/>
-      <c r="L3" s="689" t="s">
+      <c r="L3" s="708" t="s">
         <v>9</v>
       </c>
       <c r="M3" s="732" t="s">
@@ -34202,16 +34248,16 @@
       <c r="D4" s="735"/>
       <c r="E4" s="735"/>
       <c r="F4" s="735"/>
-      <c r="G4" s="582"/>
+      <c r="G4" s="601"/>
       <c r="H4" s="735" t="s">
         <v>379</v>
       </c>
       <c r="I4" s="735"/>
       <c r="J4" s="735"/>
       <c r="K4" s="735"/>
-      <c r="L4" s="580"/>
-      <c r="M4" s="581"/>
-      <c r="N4" s="691"/>
+      <c r="L4" s="599"/>
+      <c r="M4" s="600"/>
+      <c r="N4" s="710"/>
     </row>
     <row r="5" spans="1:25" ht="26">
       <c r="A5" s="730"/>
@@ -34241,9 +34287,9 @@
       <c r="K5" s="84" t="s">
         <v>113</v>
       </c>
-      <c r="L5" s="581"/>
-      <c r="M5" s="581"/>
-      <c r="N5" s="691"/>
+      <c r="L5" s="600"/>
+      <c r="M5" s="600"/>
+      <c r="N5" s="710"/>
     </row>
     <row r="6" spans="1:25" ht="84">
       <c r="A6" s="50"/>
@@ -35395,12 +35441,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>710</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="611"/>
       <c r="E1" s="388"/>
       <c r="F1" s="388"/>
       <c r="G1" s="388"/>
@@ -35450,7 +35496,7 @@
       <c r="I3" s="751"/>
       <c r="J3" s="751"/>
       <c r="K3" s="751"/>
-      <c r="L3" s="689" t="s">
+      <c r="L3" s="708" t="s">
         <v>9</v>
       </c>
       <c r="M3" s="742" t="s">
@@ -35481,7 +35527,7 @@
       <c r="K4" s="85" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="580"/>
+      <c r="L4" s="599"/>
       <c r="M4" s="743"/>
     </row>
     <row r="5" spans="1:25" ht="48">
@@ -36515,31 +36561,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>711</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="591"/>
-      <c r="K1" s="591"/>
-      <c r="L1" s="591"/>
-      <c r="M1" s="591"/>
-      <c r="N1" s="591"/>
-      <c r="O1" s="591"/>
-      <c r="P1" s="591"/>
-      <c r="Q1" s="591"/>
-      <c r="R1" s="591"/>
-      <c r="S1" s="591"/>
-      <c r="T1" s="591"/>
-      <c r="U1" s="591"/>
-      <c r="V1" s="591"/>
-      <c r="W1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="610"/>
+      <c r="K1" s="610"/>
+      <c r="L1" s="610"/>
+      <c r="M1" s="610"/>
+      <c r="N1" s="610"/>
+      <c r="O1" s="610"/>
+      <c r="P1" s="610"/>
+      <c r="Q1" s="610"/>
+      <c r="R1" s="610"/>
+      <c r="S1" s="610"/>
+      <c r="T1" s="610"/>
+      <c r="U1" s="610"/>
+      <c r="V1" s="610"/>
+      <c r="W1" s="611"/>
       <c r="X1" s="89"/>
       <c r="Y1" s="478" t="s">
         <v>7</v>
@@ -36593,16 +36639,16 @@
       <c r="P3" s="732"/>
       <c r="Q3" s="732"/>
       <c r="R3" s="732"/>
-      <c r="S3" s="689" t="s">
+      <c r="S3" s="708" t="s">
         <v>424</v>
       </c>
-      <c r="T3" s="689" t="s">
+      <c r="T3" s="708" t="s">
         <v>423</v>
       </c>
       <c r="U3" s="732" t="s">
         <v>9</v>
       </c>
-      <c r="V3" s="689" t="s">
+      <c r="V3" s="708" t="s">
         <v>425</v>
       </c>
       <c r="W3" s="733" t="s">
@@ -36632,10 +36678,10 @@
       <c r="P4" s="731"/>
       <c r="Q4" s="731"/>
       <c r="R4" s="731"/>
-      <c r="S4" s="580"/>
-      <c r="T4" s="580"/>
+      <c r="S4" s="599"/>
+      <c r="T4" s="599"/>
       <c r="U4" s="732"/>
-      <c r="V4" s="580"/>
+      <c r="V4" s="599"/>
       <c r="W4" s="733"/>
     </row>
     <row r="5" spans="1:51" ht="12" customHeight="1">
@@ -36653,32 +36699,32 @@
       </c>
       <c r="I5" s="731"/>
       <c r="J5" s="731"/>
-      <c r="K5" s="689" t="s">
+      <c r="K5" s="708" t="s">
         <v>429</v>
       </c>
       <c r="L5" s="732" t="s">
         <v>433</v>
       </c>
-      <c r="M5" s="580"/>
+      <c r="M5" s="599"/>
       <c r="N5" s="732" t="s">
         <v>430</v>
       </c>
       <c r="O5" s="732" t="s">
         <v>431</v>
       </c>
-      <c r="P5" s="689" t="s">
+      <c r="P5" s="708" t="s">
         <v>432</v>
       </c>
-      <c r="Q5" s="689" t="s">
+      <c r="Q5" s="708" t="s">
         <v>716</v>
       </c>
-      <c r="R5" s="689" t="s">
+      <c r="R5" s="708" t="s">
         <v>59</v>
       </c>
-      <c r="S5" s="580"/>
-      <c r="T5" s="580"/>
+      <c r="S5" s="599"/>
+      <c r="T5" s="599"/>
       <c r="U5" s="732"/>
-      <c r="V5" s="580"/>
+      <c r="V5" s="599"/>
       <c r="W5" s="733"/>
     </row>
     <row r="6" spans="1:51" ht="24">
@@ -36706,18 +36752,18 @@
       <c r="J6" s="218" t="s">
         <v>721</v>
       </c>
-      <c r="K6" s="581"/>
+      <c r="K6" s="600"/>
       <c r="L6" s="732"/>
-      <c r="M6" s="581"/>
+      <c r="M6" s="600"/>
       <c r="N6" s="732"/>
       <c r="O6" s="732"/>
-      <c r="P6" s="581"/>
-      <c r="Q6" s="581"/>
-      <c r="R6" s="581"/>
-      <c r="S6" s="581"/>
-      <c r="T6" s="581"/>
+      <c r="P6" s="600"/>
+      <c r="Q6" s="600"/>
+      <c r="R6" s="600"/>
+      <c r="S6" s="600"/>
+      <c r="T6" s="600"/>
       <c r="U6" s="732"/>
-      <c r="V6" s="581"/>
+      <c r="V6" s="600"/>
       <c r="W6" s="733"/>
     </row>
     <row r="7" spans="1:51" ht="48">
@@ -37972,11 +38018,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="R5:R6"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A3:A6"/>
@@ -37993,6 +38034,11 @@
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
     <mergeCell ref="K5:K6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="R5:R6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Y1" location="IDX!A1" display="IDX" xr:uid="{81941EBA-AB27-4D84-A461-A0CB925D58C9}"/>
@@ -38127,27 +38173,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>735</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="591"/>
-      <c r="K1" s="591"/>
-      <c r="L1" s="591"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="610"/>
+      <c r="K1" s="610"/>
+      <c r="L1" s="610"/>
       <c r="M1" s="753"/>
       <c r="N1" s="753"/>
       <c r="O1" s="753"/>
       <c r="P1" s="753"/>
-      <c r="Q1" s="591"/>
-      <c r="R1" s="591"/>
-      <c r="S1" s="592"/>
+      <c r="Q1" s="610"/>
+      <c r="R1" s="610"/>
+      <c r="S1" s="611"/>
       <c r="T1" s="89"/>
       <c r="U1" s="478" t="s">
         <v>7</v>
@@ -38179,15 +38225,15 @@
     <row r="3" spans="1:51" ht="12.75" customHeight="1">
       <c r="A3" s="754"/>
       <c r="B3" s="487"/>
-      <c r="C3" s="616" t="s">
+      <c r="C3" s="635" t="s">
         <v>447</v>
       </c>
-      <c r="D3" s="639"/>
-      <c r="E3" s="639"/>
-      <c r="F3" s="639"/>
-      <c r="G3" s="639"/>
-      <c r="H3" s="639"/>
-      <c r="I3" s="615"/>
+      <c r="D3" s="658"/>
+      <c r="E3" s="658"/>
+      <c r="F3" s="658"/>
+      <c r="G3" s="658"/>
+      <c r="H3" s="658"/>
+      <c r="I3" s="634"/>
       <c r="J3" s="757" t="s">
         <v>448</v>
       </c>
@@ -38196,60 +38242,60 @@
       <c r="M3" s="757"/>
       <c r="N3" s="757"/>
       <c r="O3" s="757"/>
-      <c r="P3" s="615" t="s">
+      <c r="P3" s="634" t="s">
         <v>424</v>
       </c>
-      <c r="Q3" s="615" t="s">
+      <c r="Q3" s="634" t="s">
         <v>423</v>
       </c>
-      <c r="R3" s="615" t="s">
+      <c r="R3" s="634" t="s">
         <v>9</v>
       </c>
-      <c r="S3" s="642" t="s">
+      <c r="S3" s="661" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:51" ht="10.5" customHeight="1">
       <c r="A4" s="755"/>
       <c r="B4" s="371"/>
-      <c r="C4" s="615" t="s">
+      <c r="C4" s="634" t="s">
         <v>449</v>
       </c>
-      <c r="D4" s="616" t="s">
+      <c r="D4" s="635" t="s">
         <v>694</v>
       </c>
-      <c r="E4" s="616"/>
-      <c r="F4" s="616"/>
-      <c r="G4" s="615" t="s">
+      <c r="E4" s="635"/>
+      <c r="F4" s="635"/>
+      <c r="G4" s="634" t="s">
         <v>450</v>
       </c>
-      <c r="H4" s="615" t="s">
+      <c r="H4" s="634" t="s">
         <v>423</v>
       </c>
-      <c r="I4" s="569"/>
-      <c r="J4" s="615" t="s">
+      <c r="I4" s="588"/>
+      <c r="J4" s="634" t="s">
         <v>449</v>
       </c>
-      <c r="K4" s="616" t="s">
+      <c r="K4" s="635" t="s">
         <v>694</v>
       </c>
-      <c r="L4" s="616"/>
-      <c r="M4" s="616"/>
-      <c r="N4" s="615" t="s">
+      <c r="L4" s="635"/>
+      <c r="M4" s="635"/>
+      <c r="N4" s="634" t="s">
         <v>450</v>
       </c>
-      <c r="O4" s="615" t="s">
+      <c r="O4" s="634" t="s">
         <v>423</v>
       </c>
-      <c r="P4" s="569"/>
-      <c r="Q4" s="569"/>
-      <c r="R4" s="569"/>
-      <c r="S4" s="643"/>
+      <c r="P4" s="588"/>
+      <c r="Q4" s="588"/>
+      <c r="R4" s="588"/>
+      <c r="S4" s="662"/>
     </row>
     <row r="5" spans="1:51" ht="22.75" customHeight="1">
       <c r="A5" s="756"/>
       <c r="B5" s="372"/>
-      <c r="C5" s="607"/>
+      <c r="C5" s="626"/>
       <c r="D5" s="118" t="s">
         <v>451</v>
       </c>
@@ -38259,10 +38305,10 @@
       <c r="F5" s="118" t="s">
         <v>453</v>
       </c>
-      <c r="G5" s="607"/>
-      <c r="H5" s="607"/>
-      <c r="I5" s="607"/>
-      <c r="J5" s="607"/>
+      <c r="G5" s="626"/>
+      <c r="H5" s="626"/>
+      <c r="I5" s="626"/>
+      <c r="J5" s="626"/>
       <c r="K5" s="102" t="s">
         <v>451</v>
       </c>
@@ -38272,12 +38318,12 @@
       <c r="M5" s="102" t="s">
         <v>453</v>
       </c>
-      <c r="N5" s="607"/>
-      <c r="O5" s="607"/>
-      <c r="P5" s="607"/>
-      <c r="Q5" s="607"/>
-      <c r="R5" s="607"/>
-      <c r="S5" s="644"/>
+      <c r="N5" s="626"/>
+      <c r="O5" s="626"/>
+      <c r="P5" s="626"/>
+      <c r="Q5" s="626"/>
+      <c r="R5" s="626"/>
+      <c r="S5" s="663"/>
     </row>
     <row r="6" spans="1:51" ht="96">
       <c r="A6" s="53"/>
@@ -39286,11 +39332,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="J4:J5"/>
     <mergeCell ref="K4:M4"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="A2:S2"/>
@@ -39304,6 +39345,11 @@
     <mergeCell ref="S3:S5"/>
     <mergeCell ref="N4:N5"/>
     <mergeCell ref="O4:O5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="J4:J5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U1" location="IDX!A1" display="IDX" xr:uid="{DC2A2244-E826-452B-A811-3CD065B6D100}"/>
@@ -39359,19 +39405,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" s="48" customFormat="1" ht="13">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>769</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="591"/>
-      <c r="H1" s="591"/>
-      <c r="I1" s="591"/>
-      <c r="J1" s="591"/>
-      <c r="K1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="610"/>
+      <c r="H1" s="610"/>
+      <c r="I1" s="610"/>
+      <c r="J1" s="610"/>
+      <c r="K1" s="611"/>
       <c r="L1" s="388"/>
       <c r="M1" s="388"/>
       <c r="N1" s="388"/>
@@ -39396,93 +39442,93 @@
       </c>
     </row>
     <row r="2" spans="1:31" s="26" customFormat="1">
-      <c r="A2" s="763" t="s">
+      <c r="A2" s="758" t="s">
         <v>761</v>
       </c>
-      <c r="B2" s="764"/>
-      <c r="C2" s="764"/>
-      <c r="D2" s="764"/>
-      <c r="E2" s="764"/>
-      <c r="F2" s="764"/>
-      <c r="G2" s="764"/>
-      <c r="H2" s="764"/>
-      <c r="I2" s="764"/>
-      <c r="J2" s="764"/>
-      <c r="K2" s="764"/>
-      <c r="L2" s="764"/>
-      <c r="M2" s="764"/>
-      <c r="N2" s="764"/>
-      <c r="O2" s="764"/>
-      <c r="P2" s="764"/>
-      <c r="Q2" s="764"/>
-      <c r="R2" s="764"/>
-      <c r="S2" s="764"/>
-      <c r="T2" s="764"/>
-      <c r="U2" s="764"/>
-      <c r="V2" s="764"/>
-      <c r="W2" s="764"/>
-      <c r="X2" s="764"/>
-      <c r="Y2" s="764"/>
-      <c r="Z2" s="764"/>
-      <c r="AA2" s="764"/>
-      <c r="AB2" s="764"/>
-      <c r="AC2" s="765"/>
+      <c r="B2" s="759"/>
+      <c r="C2" s="759"/>
+      <c r="D2" s="759"/>
+      <c r="E2" s="759"/>
+      <c r="F2" s="759"/>
+      <c r="G2" s="759"/>
+      <c r="H2" s="759"/>
+      <c r="I2" s="759"/>
+      <c r="J2" s="759"/>
+      <c r="K2" s="759"/>
+      <c r="L2" s="759"/>
+      <c r="M2" s="759"/>
+      <c r="N2" s="759"/>
+      <c r="O2" s="759"/>
+      <c r="P2" s="759"/>
+      <c r="Q2" s="759"/>
+      <c r="R2" s="759"/>
+      <c r="S2" s="759"/>
+      <c r="T2" s="759"/>
+      <c r="U2" s="759"/>
+      <c r="V2" s="759"/>
+      <c r="W2" s="759"/>
+      <c r="X2" s="759"/>
+      <c r="Y2" s="759"/>
+      <c r="Z2" s="759"/>
+      <c r="AA2" s="759"/>
+      <c r="AB2" s="759"/>
+      <c r="AC2" s="760"/>
       <c r="AD2" s="20"/>
       <c r="AE2" s="20"/>
     </row>
     <row r="3" spans="1:31" s="26" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A3" s="758"/>
+      <c r="A3" s="766"/>
       <c r="B3" s="488"/>
-      <c r="C3" s="760" t="s">
+      <c r="C3" s="768" t="s">
         <v>695</v>
       </c>
-      <c r="D3" s="760"/>
-      <c r="E3" s="761" t="s">
+      <c r="D3" s="768"/>
+      <c r="E3" s="764" t="s">
         <v>696</v>
       </c>
-      <c r="F3" s="761" t="s">
+      <c r="F3" s="764" t="s">
         <v>59</v>
       </c>
-      <c r="G3" s="761" t="s">
+      <c r="G3" s="764" t="s">
         <v>423</v>
       </c>
-      <c r="H3" s="761" t="s">
+      <c r="H3" s="764" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="761" t="s">
+      <c r="I3" s="764" t="s">
         <v>455</v>
       </c>
-      <c r="J3" s="761" t="s">
+      <c r="J3" s="764" t="s">
         <v>456</v>
       </c>
-      <c r="K3" s="761" t="s">
+      <c r="K3" s="764" t="s">
         <v>115</v>
       </c>
       <c r="L3" s="392"/>
       <c r="M3" s="392"/>
-      <c r="N3" s="766" t="s">
+      <c r="N3" s="761" t="s">
         <v>749</v>
       </c>
-      <c r="O3" s="766"/>
-      <c r="P3" s="766"/>
-      <c r="Q3" s="766"/>
-      <c r="R3" s="766"/>
-      <c r="S3" s="766"/>
-      <c r="T3" s="689" t="s">
+      <c r="O3" s="761"/>
+      <c r="P3" s="761"/>
+      <c r="Q3" s="761"/>
+      <c r="R3" s="761"/>
+      <c r="S3" s="761"/>
+      <c r="T3" s="708" t="s">
         <v>9</v>
       </c>
-      <c r="U3" s="767" t="s">
+      <c r="U3" s="762" t="s">
         <v>759</v>
       </c>
       <c r="V3" s="392"/>
       <c r="W3" s="392"/>
-      <c r="X3" s="766" t="s">
+      <c r="X3" s="761" t="s">
         <v>758</v>
       </c>
-      <c r="Y3" s="766"/>
-      <c r="Z3" s="766"/>
-      <c r="AA3" s="766"/>
-      <c r="AB3" s="689" t="s">
+      <c r="Y3" s="761"/>
+      <c r="Z3" s="761"/>
+      <c r="AA3" s="761"/>
+      <c r="AB3" s="708" t="s">
         <v>9</v>
       </c>
       <c r="AC3" s="742" t="s">
@@ -39492,7 +39538,7 @@
       <c r="AE3" s="20"/>
     </row>
     <row r="4" spans="1:31" s="26" customFormat="1" ht="36">
-      <c r="A4" s="759"/>
+      <c r="A4" s="767"/>
       <c r="B4" s="546"/>
       <c r="C4" s="514" t="s">
         <v>457</v>
@@ -39500,13 +39546,13 @@
       <c r="D4" s="547" t="s">
         <v>458</v>
       </c>
-      <c r="E4" s="762"/>
-      <c r="F4" s="762"/>
-      <c r="G4" s="762"/>
-      <c r="H4" s="762"/>
-      <c r="I4" s="762"/>
-      <c r="J4" s="762"/>
-      <c r="K4" s="762"/>
+      <c r="E4" s="765"/>
+      <c r="F4" s="765"/>
+      <c r="G4" s="765"/>
+      <c r="H4" s="765"/>
+      <c r="I4" s="765"/>
+      <c r="J4" s="765"/>
+      <c r="K4" s="765"/>
       <c r="L4" s="494"/>
       <c r="M4" s="494"/>
       <c r="N4" s="85" t="s">
@@ -39527,8 +39573,8 @@
       <c r="S4" s="85" t="s">
         <v>113</v>
       </c>
-      <c r="T4" s="580"/>
-      <c r="U4" s="768"/>
+      <c r="T4" s="599"/>
+      <c r="U4" s="763"/>
       <c r="V4" s="494"/>
       <c r="W4" s="494"/>
       <c r="X4" s="85" t="s">
@@ -39543,7 +39589,7 @@
       <c r="AA4" s="85" t="s">
         <v>113</v>
       </c>
-      <c r="AB4" s="580"/>
+      <c r="AB4" s="599"/>
       <c r="AC4" s="743"/>
       <c r="AD4" s="20"/>
       <c r="AE4" s="20"/>
@@ -41151,14 +41197,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="AB3:AB4"/>
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="A2:AC2"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="X3:AA3"/>
-    <mergeCell ref="K3:K4"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="C3:D3"/>
@@ -41168,6 +41206,14 @@
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="J3:J4"/>
+    <mergeCell ref="AB3:AB4"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="A2:AC2"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="X3:AA3"/>
+    <mergeCell ref="K3:K4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="AE1" location="IDX!A1" display="IDX" xr:uid="{E1A74C00-FB72-4274-834A-ADE93AE07F7F}"/>
@@ -41198,44 +41244,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="561" t="s">
+      <c r="A1" s="580" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="562"/>
-      <c r="C1" s="562"/>
-      <c r="D1" s="562"/>
-      <c r="E1" s="563"/>
+      <c r="B1" s="581"/>
+      <c r="C1" s="581"/>
+      <c r="D1" s="581"/>
+      <c r="E1" s="582"/>
       <c r="F1" s="32"/>
       <c r="G1" s="97" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="11.25" customHeight="1">
-      <c r="A2" s="564" t="s">
+      <c r="A2" s="583" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="565"/>
-      <c r="C2" s="565"/>
-      <c r="D2" s="565"/>
-      <c r="E2" s="566"/>
+      <c r="B2" s="584"/>
+      <c r="C2" s="584"/>
+      <c r="D2" s="584"/>
+      <c r="E2" s="585"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="567"/>
+      <c r="A3" s="586"/>
       <c r="B3" s="100"/>
-      <c r="C3" s="569" t="s">
+      <c r="C3" s="588" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="570" t="s">
+      <c r="D3" s="589" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="571"/>
+      <c r="E3" s="590"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="100"/>
-      <c r="C4" s="569"/>
+      <c r="C4" s="588"/>
       <c r="D4" s="100" t="s">
         <v>11</v>
       </c>
@@ -41564,44 +41610,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A1" s="572" t="s">
+      <c r="A1" s="591" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="573"/>
-      <c r="C1" s="573"/>
-      <c r="D1" s="573"/>
-      <c r="E1" s="574"/>
+      <c r="B1" s="592"/>
+      <c r="C1" s="592"/>
+      <c r="D1" s="592"/>
+      <c r="E1" s="593"/>
       <c r="G1" s="97" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="20" customFormat="1" ht="10.5" customHeight="1">
-      <c r="A2" s="575" t="s">
+      <c r="A2" s="594" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="576"/>
-      <c r="C2" s="576"/>
-      <c r="D2" s="576"/>
-      <c r="E2" s="577"/>
+      <c r="B2" s="595"/>
+      <c r="C2" s="595"/>
+      <c r="D2" s="595"/>
+      <c r="E2" s="596"/>
       <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" ht="12.5" customHeight="1">
-      <c r="A3" s="578"/>
+      <c r="A3" s="597"/>
       <c r="B3" s="85"/>
-      <c r="C3" s="580" t="s">
+      <c r="C3" s="599" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="582" t="s">
+      <c r="D3" s="601" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="583"/>
+      <c r="E3" s="602"/>
       <c r="F3" s="89"/>
       <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="579"/>
+      <c r="A4" s="598"/>
       <c r="B4" s="84"/>
-      <c r="C4" s="581"/>
+      <c r="C4" s="600"/>
       <c r="D4" s="218" t="s">
         <v>11</v>
       </c>
@@ -41990,44 +42036,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="561" t="s">
+      <c r="A1" s="580" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="562"/>
-      <c r="C1" s="562"/>
-      <c r="D1" s="562"/>
-      <c r="E1" s="563"/>
+      <c r="B1" s="581"/>
+      <c r="C1" s="581"/>
+      <c r="D1" s="581"/>
+      <c r="E1" s="582"/>
       <c r="F1" s="32"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="564" t="s">
+      <c r="A2" s="583" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="565"/>
-      <c r="C2" s="565"/>
-      <c r="D2" s="565"/>
-      <c r="E2" s="566"/>
+      <c r="B2" s="584"/>
+      <c r="C2" s="584"/>
+      <c r="D2" s="584"/>
+      <c r="E2" s="585"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="11">
-      <c r="A3" s="567"/>
+      <c r="A3" s="586"/>
       <c r="B3" s="100"/>
-      <c r="C3" s="584" t="s">
+      <c r="C3" s="603" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="570" t="s">
+      <c r="D3" s="589" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="571"/>
+      <c r="E3" s="590"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="585"/>
+      <c r="C4" s="604"/>
       <c r="D4" s="118" t="s">
         <v>11</v>
       </c>
@@ -42542,15 +42588,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="591"/>
-      <c r="F1" s="591"/>
-      <c r="G1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="610"/>
+      <c r="F1" s="610"/>
+      <c r="G1" s="611"/>
       <c r="H1" s="32"/>
       <c r="I1" s="86" t="s">
         <v>7</v>
@@ -42559,15 +42605,15 @@
       <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11" ht="26.25" customHeight="1">
-      <c r="A2" s="593" t="s">
+      <c r="A2" s="612" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="594"/>
-      <c r="C2" s="594"/>
-      <c r="D2" s="594"/>
-      <c r="E2" s="594"/>
-      <c r="F2" s="595"/>
-      <c r="G2" s="596"/>
+      <c r="B2" s="613"/>
+      <c r="C2" s="613"/>
+      <c r="D2" s="613"/>
+      <c r="E2" s="613"/>
+      <c r="F2" s="614"/>
+      <c r="G2" s="615"/>
       <c r="H2" s="32"/>
       <c r="I2" s="32"/>
       <c r="J2" s="32"/>
@@ -42576,17 +42622,17 @@
     <row r="3" spans="1:11" s="2" customFormat="1" ht="11.25" customHeight="1">
       <c r="A3" s="104"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="597" t="s">
+      <c r="C3" s="616" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="597"/>
+      <c r="D3" s="616"/>
       <c r="E3" s="122"/>
-      <c r="F3" s="597" t="s">
+      <c r="F3" s="616" t="s">
         <v>63</v>
       </c>
-      <c r="G3" s="598"/>
-      <c r="J3" s="589"/>
-      <c r="K3" s="589"/>
+      <c r="G3" s="617"/>
+      <c r="J3" s="608"/>
+      <c r="K3" s="608"/>
     </row>
     <row r="4" spans="1:11" s="2" customFormat="1" ht="11.25" customHeight="1">
       <c r="A4" s="99"/>
@@ -42604,8 +42650,8 @@
       <c r="G4" s="124" t="s">
         <v>65</v>
       </c>
-      <c r="J4" s="589"/>
-      <c r="K4" s="589"/>
+      <c r="J4" s="608"/>
+      <c r="K4" s="608"/>
     </row>
     <row r="5" spans="1:11" s="2" customFormat="1" ht="24">
       <c r="A5" s="104"/>
@@ -42804,15 +42850,15 @@
       <c r="I18"/>
     </row>
     <row r="19" spans="1:9" s="26" customFormat="1">
-      <c r="A19" s="586" t="s">
+      <c r="A19" s="605" t="s">
         <v>77</v>
       </c>
-      <c r="B19" s="587"/>
-      <c r="C19" s="587"/>
-      <c r="D19" s="587"/>
-      <c r="E19" s="587"/>
-      <c r="F19" s="587"/>
-      <c r="G19" s="588"/>
+      <c r="B19" s="606"/>
+      <c r="C19" s="606"/>
+      <c r="D19" s="606"/>
+      <c r="E19" s="606"/>
+      <c r="F19" s="606"/>
+      <c r="G19" s="607"/>
       <c r="H19" s="32"/>
       <c r="I19" s="32"/>
     </row>
@@ -43198,13 +43244,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15">
-      <c r="A1" s="590" t="s">
+      <c r="A1" s="609" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="591"/>
-      <c r="C1" s="591"/>
-      <c r="D1" s="591"/>
-      <c r="E1" s="592"/>
+      <c r="B1" s="610"/>
+      <c r="C1" s="610"/>
+      <c r="D1" s="610"/>
+      <c r="E1" s="611"/>
       <c r="F1" s="32"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
@@ -43212,25 +43258,25 @@
       <c r="H1" s="32"/>
     </row>
     <row r="2" spans="1:8" ht="14">
-      <c r="A2" s="593" t="s">
+      <c r="A2" s="612" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="594"/>
-      <c r="C2" s="595"/>
-      <c r="D2" s="595"/>
-      <c r="E2" s="596"/>
+      <c r="B2" s="613"/>
+      <c r="C2" s="614"/>
+      <c r="D2" s="614"/>
+      <c r="E2" s="615"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
       <c r="H2" s="32"/>
     </row>
     <row r="3" spans="1:8" ht="11.25" customHeight="1">
-      <c r="A3" s="600"/>
+      <c r="A3" s="619"/>
       <c r="B3" s="278"/>
-      <c r="C3" s="597" t="s">
+      <c r="C3" s="616" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="597"/>
-      <c r="E3" s="602" t="s">
+      <c r="D3" s="616"/>
+      <c r="E3" s="621" t="s">
         <v>81</v>
       </c>
       <c r="F3" s="2"/>
@@ -43238,7 +43284,7 @@
       <c r="H3" s="32"/>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="601"/>
+      <c r="A4" s="620"/>
       <c r="B4" s="252"/>
       <c r="C4" s="126" t="s">
         <v>82</v>
@@ -43246,7 +43292,7 @@
       <c r="D4" s="126" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="603"/>
+      <c r="E4" s="622"/>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" ht="24">
       <c r="A5" s="104"/>
@@ -43600,13 +43646,13 @@
       <c r="G34" s="32"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="A35" s="599" t="s">
+      <c r="A35" s="618" t="s">
         <v>120</v>
       </c>
-      <c r="B35" s="599"/>
-      <c r="C35" s="599"/>
-      <c r="D35" s="599"/>
-      <c r="E35" s="599"/>
+      <c r="B35" s="618"/>
+      <c r="C35" s="618"/>
+      <c r="D35" s="618"/>
+      <c r="E35" s="618"/>
       <c r="F35" s="32"/>
       <c r="G35" s="32"/>
       <c r="H35" s="32"/>
@@ -44070,13 +44116,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15">
-      <c r="A1" s="572" t="s">
+      <c r="A1" s="591" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="573"/>
-      <c r="C1" s="573"/>
-      <c r="D1" s="573"/>
-      <c r="E1" s="574"/>
+      <c r="B1" s="592"/>
+      <c r="C1" s="592"/>
+      <c r="D1" s="592"/>
+      <c r="E1" s="593"/>
       <c r="F1" s="32"/>
       <c r="G1" s="86" t="s">
         <v>7</v>
@@ -44093,13 +44139,13 @@
       <c r="Q1" s="32"/>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="604" t="s">
+      <c r="A2" s="623" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="605"/>
-      <c r="C2" s="605"/>
-      <c r="D2" s="605"/>
-      <c r="E2" s="606"/>
+      <c r="B2" s="624"/>
+      <c r="C2" s="624"/>
+      <c r="D2" s="624"/>
+      <c r="E2" s="625"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
       <c r="H2" s="32"/>
@@ -44114,21 +44160,21 @@
       <c r="Q2" s="32"/>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A3" s="567"/>
+      <c r="A3" s="586"/>
       <c r="B3" s="100"/>
-      <c r="C3" s="569" t="s">
+      <c r="C3" s="588" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="570" t="s">
+      <c r="D3" s="589" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="571"/>
+      <c r="E3" s="590"/>
       <c r="F3" s="130"/>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A4" s="568"/>
+      <c r="A4" s="587"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="607"/>
+      <c r="C4" s="626"/>
       <c r="D4" s="102" t="s">
         <v>11</v>
       </c>
@@ -44776,6 +44822,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EDD8FB7ED309C341A94F58A0756CD608" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="70bcba18ac9261c303654822dcc15a69">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="684e95f9-27d2-4cf0-b93c-d469076358f8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1719bfeb9034feef65d6da37310b6cc" ns2:_="">
     <xsd:import namespace="684e95f9-27d2-4cf0-b93c-d469076358f8"/>
@@ -44939,22 +45000,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{248894DE-7893-4B66-859D-8A30FCFA7578}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="684e95f9-27d2-4cf0-b93c-d469076358f8"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77665903-7C55-46FD-9DF5-09CF885D669C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3BD167C-3CD9-462B-8751-1BF2DD15E296}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44972,30 +45042,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77665903-7C55-46FD-9DF5-09CF885D669C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{248894DE-7893-4B66-859D-8A30FCFA7578}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="684e95f9-27d2-4cf0-b93c-d469076358f8"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{77410195-14e1-4fb8-904b-ab1892023667}" enabled="0" method="" siteId="{77410195-14e1-4fb8-904b-ab1892023667}" removed="1"/>

</xml_diff>